<commit_message>
BOM Economization for Bottom Board #135
</commit_message>
<xml_diff>
--- a/Deliverables/SM_Bottom Board/_BOM/eSpark BOM _Bottom (20 Boards).xlsx
+++ b/Deliverables/SM_Bottom Board/_BOM/eSpark BOM _Bottom (20 Boards).xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Faizan\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Faizan\GitHub\ColeBenson-SmartMotors\Deliverables\SM_Bottom Board\_BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -14,7 +14,7 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -88,9 +88,6 @@
     <t>CF1</t>
   </si>
   <si>
-    <t>D1, D2</t>
-  </si>
-  <si>
     <t>D12</t>
   </si>
   <si>
@@ -737,12 +734,15 @@
   </si>
   <si>
     <t>Design change required.</t>
+  </si>
+  <si>
+    <t>D1</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
   </numFmts>
@@ -916,7 +916,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -955,12 +955,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFC000"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -1203,7 +1197,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="87">
+  <cellXfs count="83">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
@@ -1379,46 +1373,16 @@
     <xf numFmtId="0" fontId="17" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="20" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="8" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="7" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1443,6 +1407,24 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1488,7 +1470,7 @@
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1787,24 +1769,24 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:R44"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="3.109375" style="25" customWidth="1"/>
-    <col min="3" max="3" width="18.6640625" style="25" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="3.140625" style="25" customWidth="1"/>
+    <col min="3" max="3" width="18.7109375" style="25" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="36" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="26.5546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="33.44140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.44140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="33.44140625" customWidth="1"/>
-    <col min="11" max="11" width="17.88671875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="20.88671875" customWidth="1"/>
-    <col min="14" max="15" width="19.109375" customWidth="1"/>
-    <col min="16" max="18" width="29.44140625" customWidth="1"/>
+    <col min="6" max="6" width="26.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="33.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="33.42578125" customWidth="1"/>
+    <col min="11" max="11" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="20.85546875" customWidth="1"/>
+    <col min="14" max="15" width="19.140625" customWidth="1"/>
+    <col min="16" max="18" width="29.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="19"/>
       <c r="C1" s="19"/>
@@ -1815,16 +1797,16 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="84"/>
-      <c r="L1" s="84"/>
-      <c r="M1" s="84"/>
-      <c r="N1" s="84"/>
-      <c r="O1" s="84"/>
-      <c r="P1" s="84"/>
-      <c r="Q1" s="84"/>
-      <c r="R1" s="84"/>
-    </row>
-    <row r="2" spans="1:18" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="K1" s="74"/>
+      <c r="L1" s="74"/>
+      <c r="M1" s="74"/>
+      <c r="N1" s="74"/>
+      <c r="O1" s="74"/>
+      <c r="P1" s="74"/>
+      <c r="Q1" s="74"/>
+      <c r="R1" s="74"/>
+    </row>
+    <row r="2" spans="1:18" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
       <c r="B2" s="20"/>
       <c r="C2" s="46"/>
@@ -1848,7 +1830,7 @@
       <c r="Q2" s="3"/>
       <c r="R2" s="43"/>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
       <c r="B3" s="21"/>
       <c r="C3" s="47"/>
@@ -1870,9 +1852,9 @@
       <c r="O3" s="4"/>
       <c r="P3" s="4"/>
       <c r="Q3" s="4"/>
-      <c r="R3" s="85"/>
-    </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="R3" s="75"/>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="21"/>
       <c r="C4" s="47"/>
@@ -1894,9 +1876,9 @@
       <c r="O4" s="6"/>
       <c r="P4" s="6"/>
       <c r="Q4" s="59"/>
-      <c r="R4" s="86"/>
-    </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="R4" s="76"/>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5" s="21"/>
       <c r="C5" s="47"/>
@@ -1918,9 +1900,9 @@
       <c r="O5" s="5"/>
       <c r="P5" s="5"/>
       <c r="Q5" s="59"/>
-      <c r="R5" s="86"/>
-    </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="R5" s="76"/>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
       <c r="B6" s="22"/>
       <c r="C6" s="48"/>
@@ -1938,9 +1920,9 @@
       <c r="O6" s="5"/>
       <c r="P6" s="5"/>
       <c r="Q6" s="59"/>
-      <c r="R6" s="86"/>
-    </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="R6" s="76"/>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
       <c r="B7" s="23"/>
       <c r="C7" s="49"/>
@@ -1958,9 +1940,9 @@
       <c r="O7" s="7"/>
       <c r="P7" s="7"/>
       <c r="Q7" s="7"/>
-      <c r="R7" s="86"/>
-    </row>
-    <row r="8" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="R7" s="76"/>
+    </row>
+    <row r="8" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
       <c r="B8" s="26"/>
       <c r="C8" s="50"/>
@@ -1978,94 +1960,94 @@
       <c r="O8" s="7"/>
       <c r="P8" s="7"/>
       <c r="Q8" s="7"/>
-      <c r="R8" s="86"/>
-    </row>
-    <row r="9" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="R8" s="76"/>
+    </row>
+    <row r="9" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
       <c r="B9" s="29" t="s">
         <v>4</v>
       </c>
       <c r="C9" s="29" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D9" s="29" t="s">
         <v>10</v>
       </c>
       <c r="E9" s="30" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F9" s="29" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G9" s="30" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H9" s="29" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="I9" s="29" t="s">
+        <v>177</v>
+      </c>
+      <c r="J9" s="29" t="s">
         <v>178</v>
       </c>
-      <c r="J9" s="29" t="s">
+      <c r="K9" s="30" t="s">
+        <v>147</v>
+      </c>
+      <c r="L9" s="29" t="s">
+        <v>162</v>
+      </c>
+      <c r="M9" s="29" t="s">
         <v>179</v>
       </c>
-      <c r="K9" s="30" t="s">
-        <v>148</v>
-      </c>
-      <c r="L9" s="29" t="s">
-        <v>163</v>
-      </c>
-      <c r="M9" s="29" t="s">
+      <c r="N9" s="29" t="s">
         <v>180</v>
       </c>
-      <c r="N9" s="29" t="s">
+      <c r="O9" s="29" t="s">
         <v>181</v>
       </c>
-      <c r="O9" s="29" t="s">
+      <c r="P9" s="29" t="s">
         <v>182</v>
       </c>
-      <c r="P9" s="29" t="s">
+      <c r="Q9" s="31" t="s">
         <v>183</v>
       </c>
-      <c r="Q9" s="31" t="s">
+      <c r="R9" s="31" t="s">
         <v>184</v>
       </c>
-      <c r="R9" s="31" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="10" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="10" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
       <c r="B10" s="53">
         <f>ROW(B10) - ROW($B$9)</f>
         <v>1</v>
       </c>
       <c r="C10" s="37" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D10" s="37" t="s">
         <v>11</v>
       </c>
       <c r="E10" s="38" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F10" s="37" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G10" s="38" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="H10" s="37" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="I10" s="37" t="s">
+        <v>185</v>
+      </c>
+      <c r="J10" s="37" t="s">
         <v>186</v>
       </c>
-      <c r="J10" s="37" t="s">
-        <v>187</v>
-      </c>
       <c r="K10" s="38" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="L10" s="37">
         <v>1</v>
@@ -2078,7 +2060,7 @@
         <v>40</v>
       </c>
       <c r="O10" s="60" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="P10" s="37">
         <v>1.9199999999999998E-2</v>
@@ -2089,38 +2071,38 @@
       </c>
       <c r="R10" s="41"/>
     </row>
-    <row r="11" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:18" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
       <c r="B11" s="53">
         <f t="shared" ref="B11:B41" si="0">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
       <c r="C11" s="39" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D11" s="39" t="s">
         <v>12</v>
       </c>
       <c r="E11" s="40" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F11" s="39" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G11" s="40" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="H11" s="39" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="I11" s="39" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="J11" s="39" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="K11" s="40" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="L11" s="39">
         <v>19</v>
@@ -2133,7 +2115,7 @@
         <v>400</v>
       </c>
       <c r="O11" s="61" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="P11" s="39">
         <v>1.4E-3</v>
@@ -2144,95 +2126,95 @@
       </c>
       <c r="R11" s="42"/>
     </row>
-    <row r="12" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
       <c r="B12" s="53">
         <f>ROW(B12) - ROW($B$9)</f>
         <v>3</v>
       </c>
-      <c r="C12" s="66" t="s">
-        <v>164</v>
-      </c>
-      <c r="D12" s="66" t="s">
+      <c r="C12" s="37" t="s">
+        <v>163</v>
+      </c>
+      <c r="D12" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="E12" s="67" t="s">
-        <v>47</v>
-      </c>
-      <c r="F12" s="66" t="s">
-        <v>175</v>
-      </c>
-      <c r="G12" s="67" t="s">
-        <v>79</v>
-      </c>
-      <c r="H12" s="66" t="s">
-        <v>128</v>
-      </c>
-      <c r="I12" s="66" t="s">
+      <c r="E12" s="38" t="s">
+        <v>46</v>
+      </c>
+      <c r="F12" s="37" t="s">
+        <v>174</v>
+      </c>
+      <c r="G12" s="38" t="s">
+        <v>78</v>
+      </c>
+      <c r="H12" s="37" t="s">
+        <v>127</v>
+      </c>
+      <c r="I12" s="37" t="s">
+        <v>189</v>
+      </c>
+      <c r="J12" s="37" t="s">
         <v>190</v>
       </c>
-      <c r="J12" s="66" t="s">
-        <v>191</v>
-      </c>
-      <c r="K12" s="67" t="s">
-        <v>151</v>
-      </c>
-      <c r="L12" s="66">
+      <c r="K12" s="38" t="s">
+        <v>150</v>
+      </c>
+      <c r="L12" s="37">
         <v>1</v>
       </c>
-      <c r="M12" s="66">
+      <c r="M12" s="37">
         <f t="shared" ref="M12:M42" si="2">L12*20</f>
         <v>20</v>
       </c>
-      <c r="N12" s="66">
+      <c r="N12" s="37">
         <v>25</v>
       </c>
-      <c r="O12" s="68" t="s">
-        <v>188</v>
-      </c>
-      <c r="P12" s="66">
+      <c r="O12" s="60" t="s">
+        <v>187</v>
+      </c>
+      <c r="P12" s="37">
         <v>6.1499999999999999E-2</v>
       </c>
-      <c r="Q12" s="69">
+      <c r="Q12" s="41">
         <f t="shared" si="1"/>
         <v>1.5375000000000001</v>
       </c>
-      <c r="R12" s="72" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="13" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="R12" s="77" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
       <c r="B13" s="53">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="C13" s="39" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D13" s="39" t="s">
         <v>14</v>
       </c>
       <c r="E13" s="40" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F13" s="39" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G13" s="40" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H13" s="39" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="I13" s="39" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="J13" s="39" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="K13" s="40" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="L13" s="39">
         <v>2</v>
@@ -2245,7 +2227,7 @@
         <v>50</v>
       </c>
       <c r="O13" s="61" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="P13" s="39">
         <v>5.0099999999999999E-2</v>
@@ -2256,38 +2238,38 @@
       </c>
       <c r="R13" s="42"/>
     </row>
-    <row r="14" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
       <c r="B14" s="53">
         <f>ROW(B14) - ROW($B$9)</f>
         <v>5</v>
       </c>
       <c r="C14" s="37" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D14" s="37" t="s">
         <v>15</v>
       </c>
       <c r="E14" s="38" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F14" s="37" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G14" s="38" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="H14" s="37" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="I14" s="37" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="J14" s="37" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="K14" s="38" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="L14" s="37">
         <v>2</v>
@@ -2300,7 +2282,7 @@
         <v>100</v>
       </c>
       <c r="O14" s="60" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="P14" s="37">
         <v>3.3999999999999998E-3</v>
@@ -2311,38 +2293,38 @@
       </c>
       <c r="R14" s="41"/>
     </row>
-    <row r="15" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
       <c r="B15" s="53">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
       <c r="C15" s="39" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D15" s="39" t="s">
         <v>16</v>
       </c>
       <c r="E15" s="40" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F15" s="39" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G15" s="40" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="H15" s="39" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="I15" s="39" t="s">
+        <v>194</v>
+      </c>
+      <c r="J15" s="39" t="s">
         <v>195</v>
       </c>
-      <c r="J15" s="39" t="s">
-        <v>196</v>
-      </c>
       <c r="K15" s="40" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="L15" s="39">
         <v>2</v>
@@ -2355,7 +2337,7 @@
         <v>50</v>
       </c>
       <c r="O15" s="61" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="P15" s="39">
         <v>7.3000000000000001E-3</v>
@@ -2366,38 +2348,38 @@
       </c>
       <c r="R15" s="42"/>
     </row>
-    <row r="16" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
       <c r="B16" s="53">
         <f>ROW(B16) - ROW($B$9)</f>
         <v>7</v>
       </c>
       <c r="C16" s="37" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D16" s="37" t="s">
         <v>17</v>
       </c>
       <c r="E16" s="38" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F16" s="37" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="G16" s="38" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="H16" s="37" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="I16" s="37" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="J16" s="37" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="K16" s="38" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="L16" s="37">
         <v>1</v>
@@ -2410,7 +2392,7 @@
         <v>40</v>
       </c>
       <c r="O16" s="60" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="P16" s="37">
         <v>1.49E-2</v>
@@ -2421,38 +2403,38 @@
       </c>
       <c r="R16" s="41"/>
     </row>
-    <row r="17" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:18" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
       <c r="B17" s="53">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
       <c r="C17" s="39" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D17" s="39" t="s">
         <v>18</v>
       </c>
       <c r="E17" s="40" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F17" s="39" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G17" s="40" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="H17" s="39" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="I17" s="39" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="J17" s="39" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="K17" s="40" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="L17" s="39">
         <v>1</v>
@@ -2465,7 +2447,7 @@
         <v>100</v>
       </c>
       <c r="O17" s="61" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="P17" s="39">
         <v>1.4E-3</v>
@@ -2476,95 +2458,95 @@
       </c>
       <c r="R17" s="42"/>
     </row>
-    <row r="18" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
       <c r="B18" s="53">
         <f>ROW(B18) - ROW($B$9)</f>
         <v>9</v>
       </c>
-      <c r="C18" s="66" t="s">
-        <v>165</v>
-      </c>
-      <c r="D18" s="66" t="s">
-        <v>19</v>
-      </c>
-      <c r="E18" s="67" t="s">
-        <v>52</v>
-      </c>
-      <c r="F18" s="66" t="s">
-        <v>175</v>
-      </c>
-      <c r="G18" s="66" t="s">
-        <v>82</v>
-      </c>
-      <c r="H18" s="66" t="s">
-        <v>132</v>
-      </c>
-      <c r="I18" s="66" t="s">
+      <c r="C18" s="37" t="s">
+        <v>164</v>
+      </c>
+      <c r="D18" s="37" t="s">
+        <v>235</v>
+      </c>
+      <c r="E18" s="38" t="s">
+        <v>51</v>
+      </c>
+      <c r="F18" s="37" t="s">
+        <v>174</v>
+      </c>
+      <c r="G18" s="37" t="s">
+        <v>81</v>
+      </c>
+      <c r="H18" s="37" t="s">
+        <v>131</v>
+      </c>
+      <c r="I18" s="37" t="s">
+        <v>197</v>
+      </c>
+      <c r="J18" s="37" t="s">
         <v>198</v>
       </c>
-      <c r="J18" s="66" t="s">
-        <v>199</v>
-      </c>
-      <c r="K18" s="67" t="s">
-        <v>186</v>
-      </c>
-      <c r="L18" s="71">
+      <c r="K18" s="38" t="s">
+        <v>185</v>
+      </c>
+      <c r="L18" s="78">
         <v>1</v>
       </c>
-      <c r="M18" s="66">
+      <c r="M18" s="37">
         <f t="shared" si="2"/>
         <v>20</v>
       </c>
-      <c r="N18" s="66">
+      <c r="N18" s="37">
         <v>25</v>
       </c>
-      <c r="O18" s="68" t="s">
-        <v>188</v>
-      </c>
-      <c r="P18" s="66">
+      <c r="O18" s="60" t="s">
+        <v>187</v>
+      </c>
+      <c r="P18" s="37">
         <v>0.17119999999999999</v>
       </c>
-      <c r="Q18" s="69">
+      <c r="Q18" s="41">
         <f t="shared" si="1"/>
         <v>4.2799999999999994</v>
       </c>
-      <c r="R18" s="72" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="19" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="R18" s="77" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="19" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
       <c r="B19" s="53">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="C19" s="39" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D19" s="39" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E19" s="40" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F19" s="39" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="G19" s="40" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="H19" s="39" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="I19" s="39" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="J19" s="39" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="K19" s="40" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="L19" s="39">
         <v>1</v>
@@ -2577,7 +2559,7 @@
         <v>25</v>
       </c>
       <c r="O19" s="61" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="P19" s="39">
         <v>0.1066</v>
@@ -2588,38 +2570,38 @@
       </c>
       <c r="R19" s="42"/>
     </row>
-    <row r="20" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
       <c r="B20" s="53">
         <f>ROW(B20) - ROW($B$9)</f>
         <v>11</v>
       </c>
       <c r="C20" s="37" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D20" s="37" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E20" s="38" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F20" s="37" t="s">
+        <v>201</v>
+      </c>
+      <c r="G20" s="38" t="s">
+        <v>83</v>
+      </c>
+      <c r="H20" s="37" t="s">
+        <v>130</v>
+      </c>
+      <c r="I20" s="37" t="s">
+        <v>185</v>
+      </c>
+      <c r="J20" s="37" t="s">
         <v>202</v>
       </c>
-      <c r="G20" s="38" t="s">
-        <v>84</v>
-      </c>
-      <c r="H20" s="37" t="s">
-        <v>131</v>
-      </c>
-      <c r="I20" s="37" t="s">
-        <v>186</v>
-      </c>
-      <c r="J20" s="37" t="s">
-        <v>203</v>
-      </c>
       <c r="K20" s="38" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="L20" s="37">
         <v>4</v>
@@ -2632,7 +2614,7 @@
         <v>100</v>
       </c>
       <c r="O20" s="60" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="P20" s="37">
         <v>2.9499999999999998E-2</v>
@@ -2643,38 +2625,38 @@
       </c>
       <c r="R20" s="41"/>
     </row>
-    <row r="21" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1"/>
       <c r="B21" s="53">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
       <c r="C21" s="39" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D21" s="39" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E21" s="40" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F21" s="39" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="G21" s="40" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H21" s="39" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="I21" s="39" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="J21" s="39" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="K21" s="40" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="L21" s="39">
         <v>1</v>
@@ -2687,7 +2669,7 @@
         <v>25</v>
       </c>
       <c r="O21" s="61" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="P21" s="39">
         <v>2.09</v>
@@ -2698,38 +2680,38 @@
       </c>
       <c r="R21" s="42"/>
     </row>
-    <row r="22" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
       <c r="B22" s="53">
         <f>ROW(B22) - ROW($B$9)</f>
         <v>13</v>
       </c>
       <c r="C22" s="37" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D22" s="37" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E22" s="38" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F22" s="37" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="G22" s="38" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="H22" s="37" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="I22" s="37" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="J22" s="37" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="K22" s="38" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="L22" s="37">
         <v>1</v>
@@ -2742,7 +2724,7 @@
         <v>25</v>
       </c>
       <c r="O22" s="60" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="P22" s="37">
         <v>9.8500000000000004E-2</v>
@@ -2753,38 +2735,38 @@
       </c>
       <c r="R22" s="41"/>
     </row>
-    <row r="23" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1"/>
       <c r="B23" s="53">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
       <c r="C23" s="39" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D23" s="39" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E23" s="40" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F23" s="39" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G23" s="40" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="H23" s="39" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="I23" s="39" t="s">
+        <v>205</v>
+      </c>
+      <c r="J23" s="39" t="s">
         <v>206</v>
       </c>
-      <c r="J23" s="39" t="s">
-        <v>207</v>
-      </c>
       <c r="K23" s="40" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="L23" s="39">
         <v>1</v>
@@ -2797,7 +2779,7 @@
         <v>30</v>
       </c>
       <c r="O23" s="61" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="P23" s="39">
         <v>4.2200000000000001E-2</v>
@@ -2808,38 +2790,38 @@
       </c>
       <c r="R23" s="42"/>
     </row>
-    <row r="24" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1"/>
       <c r="B24" s="53">
         <f>ROW(B24) - ROW($B$9)</f>
         <v>15</v>
       </c>
       <c r="C24" s="37" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D24" s="37" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E24" s="38" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F24" s="37" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="G24" s="38" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="H24" s="37" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="I24" s="37" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="J24" s="37" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="K24" s="38" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="L24" s="37">
         <v>1</v>
@@ -2852,7 +2834,7 @@
         <v>25</v>
       </c>
       <c r="O24" s="60" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="P24" s="37">
         <v>0.30840000000000001</v>
@@ -2863,38 +2845,38 @@
       </c>
       <c r="R24" s="41"/>
     </row>
-    <row r="25" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="1"/>
       <c r="B25" s="53">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
       <c r="C25" s="39" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D25" s="39" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E25" s="40" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F25" s="39" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="G25" s="40" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H25" s="39" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="I25" s="39" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="J25" s="39" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="K25" s="40" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="L25" s="39">
         <v>2</v>
@@ -2907,7 +2889,7 @@
         <v>60</v>
       </c>
       <c r="O25" s="61" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="P25" s="39">
         <v>3.4799999999999998E-2</v>
@@ -2918,38 +2900,38 @@
       </c>
       <c r="R25" s="42"/>
     </row>
-    <row r="26" spans="1:18" ht="48.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:18" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="1"/>
       <c r="B26" s="53">
         <f>ROW(B26) - ROW($B$9)</f>
         <v>17</v>
       </c>
       <c r="C26" s="37" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D26" s="37" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E26" s="38" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F26" s="37" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G26" s="38" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="H26" s="37" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="I26" s="37" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="J26" s="37" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="K26" s="38" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="L26" s="37">
         <v>40</v>
@@ -2962,7 +2944,7 @@
         <v>900</v>
       </c>
       <c r="O26" s="60" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="P26" s="37">
         <v>8.9999999999999998E-4</v>
@@ -2973,38 +2955,38 @@
       </c>
       <c r="R26" s="41"/>
     </row>
-    <row r="27" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="1"/>
       <c r="B27" s="53">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
       <c r="C27" s="39" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D27" s="39" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E27" s="40" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F27" s="39" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G27" s="40" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="H27" s="39" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="I27" s="39" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="J27" s="39" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="K27" s="40" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="L27" s="39">
         <v>7</v>
@@ -3017,7 +2999,7 @@
         <v>200</v>
       </c>
       <c r="O27" s="61" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="P27" s="39">
         <v>1.1999999999999999E-3</v>
@@ -3028,38 +3010,38 @@
       </c>
       <c r="R27" s="42"/>
     </row>
-    <row r="28" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
       <c r="B28" s="53">
         <f>ROW(B28) - ROW($B$9)</f>
         <v>19</v>
       </c>
       <c r="C28" s="37" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D28" s="37" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E28" s="38" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F28" s="37" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G28" s="38" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="H28" s="37" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="I28" s="37" t="s">
+        <v>211</v>
+      </c>
+      <c r="J28" s="37" t="s">
         <v>212</v>
       </c>
-      <c r="J28" s="37" t="s">
-        <v>213</v>
-      </c>
       <c r="K28" s="38" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L28" s="37">
         <v>1</v>
@@ -3072,7 +3054,7 @@
         <v>100</v>
       </c>
       <c r="O28" s="60" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="P28" s="37">
         <v>2.0999999999999999E-3</v>
@@ -3083,38 +3065,38 @@
       </c>
       <c r="R28" s="41"/>
     </row>
-    <row r="29" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:18" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1"/>
       <c r="B29" s="53">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="C29" s="39" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D29" s="39" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E29" s="40" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F29" s="39" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G29" s="40" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="H29" s="39" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="I29" s="39" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="J29" s="39" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="K29" s="40" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="L29" s="39">
         <v>2</v>
@@ -3127,7 +3109,7 @@
         <v>100</v>
       </c>
       <c r="O29" s="61" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="P29" s="39">
         <v>1.4E-3</v>
@@ -3138,38 +3120,38 @@
       </c>
       <c r="R29" s="42"/>
     </row>
-    <row r="30" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:18" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1"/>
       <c r="B30" s="53">
         <f>ROW(B30) - ROW($B$9)</f>
         <v>21</v>
       </c>
       <c r="C30" s="37" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D30" s="37" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E30" s="38" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F30" s="37" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G30" s="38" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H30" s="37" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="I30" s="37" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="J30" s="37" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="K30" s="38" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="L30" s="37">
         <v>1</v>
@@ -3182,7 +3164,7 @@
         <v>100</v>
       </c>
       <c r="O30" s="60" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="P30" s="37">
         <v>1.4E-3</v>
@@ -3193,38 +3175,38 @@
       </c>
       <c r="R30" s="41"/>
     </row>
-    <row r="31" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1"/>
       <c r="B31" s="53">
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
       <c r="C31" s="39" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D31" s="39" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E31" s="40" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F31" s="39" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="G31" s="40" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="H31" s="39" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="I31" s="39" t="s">
+        <v>215</v>
+      </c>
+      <c r="J31" s="39" t="s">
         <v>216</v>
       </c>
-      <c r="J31" s="39" t="s">
-        <v>217</v>
-      </c>
       <c r="K31" s="40" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="L31" s="39">
         <v>2</v>
@@ -3237,7 +3219,7 @@
         <v>50</v>
       </c>
       <c r="O31" s="61" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="P31" s="39">
         <v>1.01E-2</v>
@@ -3248,266 +3230,266 @@
       </c>
       <c r="R31" s="42"/>
     </row>
-    <row r="32" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1"/>
       <c r="B32" s="53">
         <f>ROW(B32) - ROW($B$9)</f>
         <v>23</v>
       </c>
-      <c r="C32" s="73" t="s">
-        <v>92</v>
-      </c>
-      <c r="D32" s="73" t="s">
-        <v>33</v>
-      </c>
-      <c r="E32" s="74" t="s">
-        <v>66</v>
-      </c>
-      <c r="F32" s="73" t="s">
-        <v>92</v>
-      </c>
-      <c r="G32" s="74" t="s">
-        <v>186</v>
-      </c>
-      <c r="H32" s="73" t="s">
-        <v>186</v>
-      </c>
-      <c r="I32" s="73" t="s">
-        <v>186</v>
-      </c>
-      <c r="J32" s="73" t="s">
-        <v>186</v>
-      </c>
-      <c r="K32" s="74" t="s">
-        <v>186</v>
-      </c>
-      <c r="L32" s="73">
+      <c r="C32" s="67" t="s">
+        <v>91</v>
+      </c>
+      <c r="D32" s="67" t="s">
+        <v>32</v>
+      </c>
+      <c r="E32" s="68" t="s">
+        <v>65</v>
+      </c>
+      <c r="F32" s="67" t="s">
+        <v>91</v>
+      </c>
+      <c r="G32" s="68" t="s">
+        <v>185</v>
+      </c>
+      <c r="H32" s="67" t="s">
+        <v>185</v>
+      </c>
+      <c r="I32" s="67" t="s">
+        <v>185</v>
+      </c>
+      <c r="J32" s="67" t="s">
+        <v>185</v>
+      </c>
+      <c r="K32" s="68" t="s">
+        <v>185</v>
+      </c>
+      <c r="L32" s="67">
         <v>8</v>
       </c>
-      <c r="M32" s="73">
+      <c r="M32" s="67">
         <f t="shared" si="2"/>
         <v>160</v>
       </c>
-      <c r="N32" s="73">
+      <c r="N32" s="67">
         <v>160</v>
       </c>
-      <c r="O32" s="73" t="s">
-        <v>186</v>
-      </c>
-      <c r="P32" s="73">
+      <c r="O32" s="67" t="s">
+        <v>185</v>
+      </c>
+      <c r="P32" s="67">
         <v>0</v>
       </c>
-      <c r="Q32" s="75">
+      <c r="Q32" s="69">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="R32" s="75" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="33" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="R32" s="69" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="33" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="1"/>
       <c r="B33" s="53">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="C33" s="76" t="s">
-        <v>172</v>
-      </c>
-      <c r="D33" s="76" t="s">
-        <v>34</v>
-      </c>
-      <c r="E33" s="77" t="s">
-        <v>67</v>
-      </c>
-      <c r="F33" s="76" t="s">
-        <v>175</v>
-      </c>
-      <c r="G33" s="77" t="s">
-        <v>93</v>
-      </c>
-      <c r="H33" s="76" t="s">
-        <v>140</v>
-      </c>
-      <c r="I33" s="76" t="s">
+      <c r="C33" s="79" t="s">
+        <v>171</v>
+      </c>
+      <c r="D33" s="79" t="s">
+        <v>33</v>
+      </c>
+      <c r="E33" s="80" t="s">
+        <v>66</v>
+      </c>
+      <c r="F33" s="79" t="s">
+        <v>174</v>
+      </c>
+      <c r="G33" s="80" t="s">
+        <v>92</v>
+      </c>
+      <c r="H33" s="79" t="s">
+        <v>139</v>
+      </c>
+      <c r="I33" s="79" t="s">
+        <v>218</v>
+      </c>
+      <c r="J33" s="79" t="s">
         <v>219</v>
       </c>
-      <c r="J33" s="76" t="s">
-        <v>220</v>
-      </c>
-      <c r="K33" s="77" t="s">
-        <v>186</v>
-      </c>
-      <c r="L33" s="76">
+      <c r="K33" s="80" t="s">
+        <v>185</v>
+      </c>
+      <c r="L33" s="79">
         <v>1</v>
       </c>
-      <c r="M33" s="76">
+      <c r="M33" s="79">
         <f t="shared" si="2"/>
         <v>20</v>
       </c>
-      <c r="N33" s="76">
+      <c r="N33" s="79">
         <v>30</v>
       </c>
-      <c r="O33" s="78" t="s">
-        <v>188</v>
-      </c>
-      <c r="P33" s="76">
+      <c r="O33" s="81" t="s">
+        <v>187</v>
+      </c>
+      <c r="P33" s="79">
         <v>4.9599999999999998E-2</v>
       </c>
-      <c r="Q33" s="79">
+      <c r="Q33" s="82">
         <f t="shared" si="1"/>
         <v>1.488</v>
       </c>
-      <c r="R33" s="70" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="34" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="R33" s="77" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="34" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1"/>
       <c r="B34" s="53">
         <f>ROW(B34) - ROW($B$9)</f>
         <v>25</v>
       </c>
-      <c r="C34" s="62" t="s">
-        <v>173</v>
-      </c>
-      <c r="D34" s="62" t="s">
-        <v>35</v>
-      </c>
-      <c r="E34" s="63" t="s">
-        <v>68</v>
-      </c>
-      <c r="F34" s="62" t="s">
-        <v>176</v>
-      </c>
-      <c r="G34" s="63" t="s">
-        <v>119</v>
-      </c>
-      <c r="H34" s="62" t="s">
-        <v>141</v>
-      </c>
-      <c r="I34" s="62" t="s">
+      <c r="C34" s="37" t="s">
+        <v>172</v>
+      </c>
+      <c r="D34" s="37" t="s">
+        <v>34</v>
+      </c>
+      <c r="E34" s="38" t="s">
+        <v>67</v>
+      </c>
+      <c r="F34" s="37" t="s">
+        <v>175</v>
+      </c>
+      <c r="G34" s="38" t="s">
+        <v>118</v>
+      </c>
+      <c r="H34" s="37" t="s">
+        <v>140</v>
+      </c>
+      <c r="I34" s="37" t="s">
+        <v>220</v>
+      </c>
+      <c r="J34" s="37" t="s">
         <v>221</v>
       </c>
-      <c r="J34" s="62" t="s">
-        <v>222</v>
-      </c>
-      <c r="K34" s="63" t="s">
-        <v>186</v>
-      </c>
-      <c r="L34" s="62">
+      <c r="K34" s="38" t="s">
+        <v>185</v>
+      </c>
+      <c r="L34" s="37">
         <v>1</v>
       </c>
-      <c r="M34" s="62">
+      <c r="M34" s="37">
         <f t="shared" si="2"/>
         <v>20</v>
       </c>
-      <c r="N34" s="62">
+      <c r="N34" s="37">
         <v>22</v>
       </c>
-      <c r="O34" s="64" t="s">
-        <v>188</v>
-      </c>
-      <c r="P34" s="62">
+      <c r="O34" s="60" t="s">
+        <v>187</v>
+      </c>
+      <c r="P34" s="37">
         <v>10.947699999999999</v>
       </c>
-      <c r="Q34" s="65">
+      <c r="Q34" s="41">
         <f t="shared" si="1"/>
         <v>240.84939999999997</v>
       </c>
-      <c r="R34" s="70" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="35" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="R34" s="77" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="35" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="1"/>
       <c r="B35" s="53">
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
-      <c r="C35" s="76" t="s">
-        <v>173</v>
-      </c>
-      <c r="D35" s="76" t="s">
-        <v>36</v>
-      </c>
-      <c r="E35" s="77" t="s">
-        <v>69</v>
-      </c>
-      <c r="F35" s="76" t="s">
-        <v>94</v>
-      </c>
-      <c r="G35" s="77" t="s">
-        <v>120</v>
-      </c>
-      <c r="H35" s="76" t="s">
-        <v>142</v>
-      </c>
-      <c r="I35" s="76" t="s">
+      <c r="C35" s="79" t="s">
+        <v>172</v>
+      </c>
+      <c r="D35" s="79" t="s">
+        <v>35</v>
+      </c>
+      <c r="E35" s="80" t="s">
+        <v>68</v>
+      </c>
+      <c r="F35" s="79" t="s">
+        <v>93</v>
+      </c>
+      <c r="G35" s="80" t="s">
+        <v>119</v>
+      </c>
+      <c r="H35" s="79" t="s">
+        <v>141</v>
+      </c>
+      <c r="I35" s="79" t="s">
+        <v>223</v>
+      </c>
+      <c r="J35" s="79" t="s">
         <v>224</v>
       </c>
-      <c r="J35" s="76" t="s">
-        <v>225</v>
-      </c>
-      <c r="K35" s="77" t="s">
-        <v>186</v>
-      </c>
-      <c r="L35" s="76">
+      <c r="K35" s="80" t="s">
+        <v>185</v>
+      </c>
+      <c r="L35" s="79">
         <v>1</v>
       </c>
-      <c r="M35" s="76">
+      <c r="M35" s="79">
         <f t="shared" si="2"/>
         <v>20</v>
       </c>
-      <c r="N35" s="76">
+      <c r="N35" s="79">
         <v>22</v>
       </c>
-      <c r="O35" s="78" t="s">
-        <v>188</v>
-      </c>
-      <c r="P35" s="76">
+      <c r="O35" s="81" t="s">
+        <v>187</v>
+      </c>
+      <c r="P35" s="79">
         <v>3.0078999999999998</v>
       </c>
-      <c r="Q35" s="79">
+      <c r="Q35" s="82">
         <f t="shared" si="1"/>
         <v>66.1738</v>
       </c>
-      <c r="R35" s="70" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="36" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="R35" s="77" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="36" spans="1:18" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="1"/>
       <c r="B36" s="53">
         <f>ROW(B36) - ROW($B$9)</f>
         <v>27</v>
       </c>
       <c r="C36" s="62" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D36" s="62" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E36" s="63" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="F36" s="62" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="G36" s="63" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="H36" s="62" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="I36" s="62" t="s">
+        <v>225</v>
+      </c>
+      <c r="J36" s="62" t="s">
         <v>226</v>
       </c>
-      <c r="J36" s="62" t="s">
-        <v>227</v>
-      </c>
       <c r="K36" s="63" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="L36" s="62">
         <v>1</v>
@@ -3520,7 +3502,7 @@
         <v>22</v>
       </c>
       <c r="O36" s="64" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="P36" s="62">
         <v>4.2937000000000003</v>
@@ -3529,42 +3511,42 @@
         <f t="shared" si="1"/>
         <v>94.461400000000012</v>
       </c>
-      <c r="R36" s="70" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="37" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="R36" s="66" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="37" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="1"/>
       <c r="B37" s="53">
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
       <c r="C37" s="39" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D37" s="39" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E37" s="40" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="F37" s="39" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G37" s="40" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H37" s="39" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I37" s="39" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="J37" s="39" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="K37" s="40" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="L37" s="39">
         <v>1</v>
@@ -3577,7 +3559,7 @@
         <v>22</v>
       </c>
       <c r="O37" s="61" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="P37" s="39">
         <v>10.6416</v>
@@ -3588,38 +3570,38 @@
       </c>
       <c r="R37" s="42"/>
     </row>
-    <row r="38" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="1"/>
       <c r="B38" s="53">
         <f>ROW(B38) - ROW($B$9)</f>
         <v>29</v>
       </c>
       <c r="C38" s="37" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D38" s="37" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E38" s="38" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="F38" s="37" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="G38" s="38" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="H38" s="37" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="I38" s="37" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="J38" s="37" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="K38" s="38" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="L38" s="37">
         <v>1</v>
@@ -3632,7 +3614,7 @@
         <v>22</v>
       </c>
       <c r="O38" s="60" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="P38" s="37">
         <v>0.3337</v>
@@ -3643,38 +3625,38 @@
       </c>
       <c r="R38" s="41"/>
     </row>
-    <row r="39" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="1"/>
       <c r="B39" s="53">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
       <c r="C39" s="39" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D39" s="39" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E39" s="40" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="F39" s="39" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G39" s="40" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="H39" s="39" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="I39" s="39" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="J39" s="39" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="K39" s="40" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="L39" s="39">
         <v>1</v>
@@ -3687,7 +3669,7 @@
         <v>22</v>
       </c>
       <c r="O39" s="61" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="P39" s="39">
         <v>1.06</v>
@@ -3698,38 +3680,38 @@
       </c>
       <c r="R39" s="42"/>
     </row>
-    <row r="40" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="1"/>
       <c r="B40" s="53">
         <f>ROW(B40) - ROW($B$9)</f>
         <v>31</v>
       </c>
       <c r="C40" s="37" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D40" s="37" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E40" s="38" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="F40" s="37" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="G40" s="38" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="H40" s="37" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="I40" s="37" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="J40" s="37" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="K40" s="38" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="L40" s="37">
         <v>1</v>
@@ -3742,7 +3724,7 @@
         <v>22</v>
       </c>
       <c r="O40" s="60" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="P40" s="37">
         <v>0.77</v>
@@ -3753,38 +3735,38 @@
       </c>
       <c r="R40" s="41"/>
     </row>
-    <row r="41" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="1"/>
       <c r="B41" s="53">
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
       <c r="C41" s="39" t="s">
+        <v>173</v>
+      </c>
+      <c r="D41" s="39" t="s">
+        <v>41</v>
+      </c>
+      <c r="E41" s="40" t="s">
+        <v>74</v>
+      </c>
+      <c r="F41" s="39" t="s">
         <v>174</v>
       </c>
-      <c r="D41" s="39" t="s">
-        <v>42</v>
-      </c>
-      <c r="E41" s="40" t="s">
-        <v>75</v>
-      </c>
-      <c r="F41" s="39" t="s">
-        <v>175</v>
-      </c>
       <c r="G41" s="40" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H41" s="39" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I41" s="39" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="J41" s="39" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="K41" s="40" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="L41" s="39">
         <v>1</v>
@@ -3797,7 +3779,7 @@
         <v>22</v>
       </c>
       <c r="O41" s="61" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="P41" s="39">
         <v>0.499</v>
@@ -3808,38 +3790,38 @@
       </c>
       <c r="R41" s="42"/>
     </row>
-    <row r="42" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="1"/>
       <c r="B42" s="53">
         <f>ROW(B42) - ROW($B$9)</f>
         <v>33</v>
       </c>
       <c r="C42" s="37" t="s">
+        <v>173</v>
+      </c>
+      <c r="D42" s="37" t="s">
+        <v>42</v>
+      </c>
+      <c r="E42" s="38" t="s">
+        <v>75</v>
+      </c>
+      <c r="F42" s="37" t="s">
         <v>174</v>
       </c>
-      <c r="D42" s="37" t="s">
-        <v>43</v>
-      </c>
-      <c r="E42" s="38" t="s">
-        <v>76</v>
-      </c>
-      <c r="F42" s="37" t="s">
-        <v>175</v>
-      </c>
       <c r="G42" s="38" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="H42" s="37" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="I42" s="37" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="J42" s="58" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="K42" s="38" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="L42" s="37">
         <v>1</v>
@@ -3852,7 +3834,7 @@
         <v>22</v>
       </c>
       <c r="O42" s="60" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="P42" s="37">
         <v>0.69</v>
@@ -3863,7 +3845,7 @@
       </c>
       <c r="R42" s="41"/>
     </row>
-    <row r="43" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A43" s="1"/>
       <c r="B43" s="32"/>
       <c r="C43" s="51"/>
@@ -3880,17 +3862,17 @@
       <c r="L43" s="36"/>
       <c r="M43" s="36"/>
       <c r="N43" s="36"/>
-      <c r="O43" s="80" t="s">
-        <v>233</v>
-      </c>
-      <c r="P43" s="81"/>
-      <c r="Q43" s="80">
+      <c r="O43" s="70" t="s">
+        <v>232</v>
+      </c>
+      <c r="P43" s="71"/>
+      <c r="Q43" s="70">
         <f>SUM(Q10:Q42)</f>
         <v>795.37520000000006</v>
       </c>
       <c r="R43" s="44"/>
     </row>
-    <row r="44" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="1"/>
       <c r="B44" s="24"/>
       <c r="C44" s="52"/>
@@ -3907,11 +3889,11 @@
       <c r="L44" s="9"/>
       <c r="M44" s="9"/>
       <c r="N44" s="9"/>
-      <c r="O44" s="82" t="s">
-        <v>234</v>
-      </c>
-      <c r="P44" s="83"/>
-      <c r="Q44" s="82">
+      <c r="O44" s="72" t="s">
+        <v>233</v>
+      </c>
+      <c r="P44" s="73"/>
+      <c r="Q44" s="72">
         <f>Q43/20</f>
         <v>39.76876</v>
       </c>

</xml_diff>

<commit_message>
Schematic changes for Bottom Board #135
</commit_message>
<xml_diff>
--- a/Deliverables/SM_Bottom Board/_BOM/eSpark BOM _Bottom (20 Boards).xlsx
+++ b/Deliverables/SM_Bottom Board/_BOM/eSpark BOM _Bottom (20 Boards).xlsx
@@ -916,7 +916,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -949,12 +949,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -1197,7 +1191,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="83">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
@@ -1361,28 +1355,13 @@
     <xf numFmtId="0" fontId="18" fillId="4" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="7" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1414,16 +1393,7 @@
     <xf numFmtId="0" fontId="21" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1797,14 +1767,14 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="74"/>
-      <c r="L1" s="74"/>
-      <c r="M1" s="74"/>
-      <c r="N1" s="74"/>
-      <c r="O1" s="74"/>
-      <c r="P1" s="74"/>
-      <c r="Q1" s="74"/>
-      <c r="R1" s="74"/>
+      <c r="K1" s="69"/>
+      <c r="L1" s="69"/>
+      <c r="M1" s="69"/>
+      <c r="N1" s="69"/>
+      <c r="O1" s="69"/>
+      <c r="P1" s="69"/>
+      <c r="Q1" s="69"/>
+      <c r="R1" s="69"/>
     </row>
     <row r="2" spans="1:18" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1852,7 +1822,7 @@
       <c r="O3" s="4"/>
       <c r="P3" s="4"/>
       <c r="Q3" s="4"/>
-      <c r="R3" s="75"/>
+      <c r="R3" s="70"/>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -1876,7 +1846,7 @@
       <c r="O4" s="6"/>
       <c r="P4" s="6"/>
       <c r="Q4" s="59"/>
-      <c r="R4" s="76"/>
+      <c r="R4" s="71"/>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -1900,7 +1870,7 @@
       <c r="O5" s="5"/>
       <c r="P5" s="5"/>
       <c r="Q5" s="59"/>
-      <c r="R5" s="76"/>
+      <c r="R5" s="71"/>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -1920,7 +1890,7 @@
       <c r="O6" s="5"/>
       <c r="P6" s="5"/>
       <c r="Q6" s="59"/>
-      <c r="R6" s="76"/>
+      <c r="R6" s="71"/>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -1940,7 +1910,7 @@
       <c r="O7" s="7"/>
       <c r="P7" s="7"/>
       <c r="Q7" s="7"/>
-      <c r="R7" s="76"/>
+      <c r="R7" s="71"/>
     </row>
     <row r="8" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -1960,7 +1930,7 @@
       <c r="O8" s="7"/>
       <c r="P8" s="7"/>
       <c r="Q8" s="7"/>
-      <c r="R8" s="76"/>
+      <c r="R8" s="71"/>
     </row>
     <row r="9" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -2179,7 +2149,7 @@
         <f t="shared" si="1"/>
         <v>1.5375000000000001</v>
       </c>
-      <c r="R12" s="77" t="s">
+      <c r="R12" s="72" t="s">
         <v>191</v>
       </c>
     </row>
@@ -2491,7 +2461,7 @@
       <c r="K18" s="38" t="s">
         <v>185</v>
       </c>
-      <c r="L18" s="78">
+      <c r="L18" s="73">
         <v>1</v>
       </c>
       <c r="M18" s="37">
@@ -2511,7 +2481,7 @@
         <f t="shared" si="1"/>
         <v>4.2799999999999994</v>
       </c>
-      <c r="R18" s="77" t="s">
+      <c r="R18" s="72" t="s">
         <v>199</v>
       </c>
     </row>
@@ -3236,54 +3206,54 @@
         <f>ROW(B32) - ROW($B$9)</f>
         <v>23</v>
       </c>
-      <c r="C32" s="67" t="s">
+      <c r="C32" s="62" t="s">
         <v>91</v>
       </c>
-      <c r="D32" s="67" t="s">
+      <c r="D32" s="62" t="s">
         <v>32</v>
       </c>
-      <c r="E32" s="68" t="s">
+      <c r="E32" s="63" t="s">
         <v>65</v>
       </c>
-      <c r="F32" s="67" t="s">
+      <c r="F32" s="62" t="s">
         <v>91</v>
       </c>
-      <c r="G32" s="68" t="s">
-        <v>185</v>
-      </c>
-      <c r="H32" s="67" t="s">
-        <v>185</v>
-      </c>
-      <c r="I32" s="67" t="s">
-        <v>185</v>
-      </c>
-      <c r="J32" s="67" t="s">
-        <v>185</v>
-      </c>
-      <c r="K32" s="68" t="s">
-        <v>185</v>
-      </c>
-      <c r="L32" s="67">
+      <c r="G32" s="63" t="s">
+        <v>185</v>
+      </c>
+      <c r="H32" s="62" t="s">
+        <v>185</v>
+      </c>
+      <c r="I32" s="62" t="s">
+        <v>185</v>
+      </c>
+      <c r="J32" s="62" t="s">
+        <v>185</v>
+      </c>
+      <c r="K32" s="63" t="s">
+        <v>185</v>
+      </c>
+      <c r="L32" s="62">
         <v>8</v>
       </c>
-      <c r="M32" s="67">
+      <c r="M32" s="62">
         <f t="shared" si="2"/>
         <v>160</v>
       </c>
-      <c r="N32" s="67">
+      <c r="N32" s="62">
         <v>160</v>
       </c>
-      <c r="O32" s="67" t="s">
-        <v>185</v>
-      </c>
-      <c r="P32" s="67">
+      <c r="O32" s="62" t="s">
+        <v>185</v>
+      </c>
+      <c r="P32" s="62">
         <v>0</v>
       </c>
-      <c r="Q32" s="69">
+      <c r="Q32" s="64">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="R32" s="69" t="s">
+      <c r="R32" s="64" t="s">
         <v>217</v>
       </c>
     </row>
@@ -3293,54 +3263,54 @@
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="C33" s="79" t="s">
+      <c r="C33" s="39" t="s">
         <v>171</v>
       </c>
-      <c r="D33" s="79" t="s">
+      <c r="D33" s="39" t="s">
         <v>33</v>
       </c>
-      <c r="E33" s="80" t="s">
+      <c r="E33" s="40" t="s">
         <v>66</v>
       </c>
-      <c r="F33" s="79" t="s">
+      <c r="F33" s="39" t="s">
         <v>174</v>
       </c>
-      <c r="G33" s="80" t="s">
+      <c r="G33" s="40" t="s">
         <v>92</v>
       </c>
-      <c r="H33" s="79" t="s">
+      <c r="H33" s="39" t="s">
         <v>139</v>
       </c>
-      <c r="I33" s="79" t="s">
+      <c r="I33" s="39" t="s">
         <v>218</v>
       </c>
-      <c r="J33" s="79" t="s">
+      <c r="J33" s="39" t="s">
         <v>219</v>
       </c>
-      <c r="K33" s="80" t="s">
-        <v>185</v>
-      </c>
-      <c r="L33" s="79">
+      <c r="K33" s="40" t="s">
+        <v>185</v>
+      </c>
+      <c r="L33" s="39">
         <v>1</v>
       </c>
-      <c r="M33" s="79">
+      <c r="M33" s="39">
         <f t="shared" si="2"/>
         <v>20</v>
       </c>
-      <c r="N33" s="79">
+      <c r="N33" s="39">
         <v>30</v>
       </c>
-      <c r="O33" s="81" t="s">
+      <c r="O33" s="61" t="s">
         <v>187</v>
       </c>
-      <c r="P33" s="79">
+      <c r="P33" s="39">
         <v>4.9599999999999998E-2</v>
       </c>
-      <c r="Q33" s="82">
+      <c r="Q33" s="42">
         <f t="shared" si="1"/>
         <v>1.488</v>
       </c>
-      <c r="R33" s="77" t="s">
+      <c r="R33" s="74" t="s">
         <v>234</v>
       </c>
     </row>
@@ -3397,7 +3367,7 @@
         <f t="shared" si="1"/>
         <v>240.84939999999997</v>
       </c>
-      <c r="R34" s="77" t="s">
+      <c r="R34" s="72" t="s">
         <v>222</v>
       </c>
     </row>
@@ -3407,54 +3377,54 @@
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
-      <c r="C35" s="79" t="s">
+      <c r="C35" s="39" t="s">
         <v>172</v>
       </c>
-      <c r="D35" s="79" t="s">
+      <c r="D35" s="39" t="s">
         <v>35</v>
       </c>
-      <c r="E35" s="80" t="s">
+      <c r="E35" s="40" t="s">
         <v>68</v>
       </c>
-      <c r="F35" s="79" t="s">
+      <c r="F35" s="39" t="s">
         <v>93</v>
       </c>
-      <c r="G35" s="80" t="s">
+      <c r="G35" s="40" t="s">
         <v>119</v>
       </c>
-      <c r="H35" s="79" t="s">
+      <c r="H35" s="39" t="s">
         <v>141</v>
       </c>
-      <c r="I35" s="79" t="s">
+      <c r="I35" s="39" t="s">
         <v>223</v>
       </c>
-      <c r="J35" s="79" t="s">
+      <c r="J35" s="39" t="s">
         <v>224</v>
       </c>
-      <c r="K35" s="80" t="s">
-        <v>185</v>
-      </c>
-      <c r="L35" s="79">
+      <c r="K35" s="40" t="s">
+        <v>185</v>
+      </c>
+      <c r="L35" s="39">
         <v>1</v>
       </c>
-      <c r="M35" s="79">
+      <c r="M35" s="39">
         <f t="shared" si="2"/>
         <v>20</v>
       </c>
-      <c r="N35" s="79">
+      <c r="N35" s="39">
         <v>22</v>
       </c>
-      <c r="O35" s="81" t="s">
+      <c r="O35" s="61" t="s">
         <v>187</v>
       </c>
-      <c r="P35" s="79">
+      <c r="P35" s="39">
         <v>3.0078999999999998</v>
       </c>
-      <c r="Q35" s="82">
+      <c r="Q35" s="42">
         <f t="shared" si="1"/>
         <v>66.1738</v>
       </c>
-      <c r="R35" s="77" t="s">
+      <c r="R35" s="74" t="s">
         <v>222</v>
       </c>
     </row>
@@ -3464,54 +3434,54 @@
         <f>ROW(B36) - ROW($B$9)</f>
         <v>27</v>
       </c>
-      <c r="C36" s="62" t="s">
+      <c r="C36" s="37" t="s">
         <v>172</v>
       </c>
-      <c r="D36" s="62" t="s">
+      <c r="D36" s="37" t="s">
         <v>36</v>
       </c>
-      <c r="E36" s="63" t="s">
+      <c r="E36" s="38" t="s">
         <v>69</v>
       </c>
-      <c r="F36" s="62" t="s">
+      <c r="F36" s="37" t="s">
         <v>94</v>
       </c>
-      <c r="G36" s="63" t="s">
+      <c r="G36" s="38" t="s">
         <v>120</v>
       </c>
-      <c r="H36" s="62" t="s">
+      <c r="H36" s="37" t="s">
         <v>142</v>
       </c>
-      <c r="I36" s="62" t="s">
+      <c r="I36" s="37" t="s">
         <v>225</v>
       </c>
-      <c r="J36" s="62" t="s">
+      <c r="J36" s="37" t="s">
         <v>226</v>
       </c>
-      <c r="K36" s="63" t="s">
-        <v>185</v>
-      </c>
-      <c r="L36" s="62">
+      <c r="K36" s="38" t="s">
+        <v>185</v>
+      </c>
+      <c r="L36" s="37">
         <v>1</v>
       </c>
-      <c r="M36" s="62">
+      <c r="M36" s="37">
         <f t="shared" si="2"/>
         <v>20</v>
       </c>
-      <c r="N36" s="62">
+      <c r="N36" s="37">
         <v>22</v>
       </c>
-      <c r="O36" s="64" t="s">
+      <c r="O36" s="60" t="s">
         <v>187</v>
       </c>
-      <c r="P36" s="62">
+      <c r="P36" s="37">
         <v>4.2937000000000003</v>
       </c>
-      <c r="Q36" s="65">
+      <c r="Q36" s="41">
         <f t="shared" si="1"/>
         <v>94.461400000000012</v>
       </c>
-      <c r="R36" s="66" t="s">
+      <c r="R36" s="72" t="s">
         <v>227</v>
       </c>
     </row>
@@ -3862,11 +3832,11 @@
       <c r="L43" s="36"/>
       <c r="M43" s="36"/>
       <c r="N43" s="36"/>
-      <c r="O43" s="70" t="s">
+      <c r="O43" s="65" t="s">
         <v>232</v>
       </c>
-      <c r="P43" s="71"/>
-      <c r="Q43" s="70">
+      <c r="P43" s="66"/>
+      <c r="Q43" s="65">
         <f>SUM(Q10:Q42)</f>
         <v>795.37520000000006</v>
       </c>
@@ -3889,11 +3859,11 @@
       <c r="L44" s="9"/>
       <c r="M44" s="9"/>
       <c r="N44" s="9"/>
-      <c r="O44" s="72" t="s">
+      <c r="O44" s="67" t="s">
         <v>233</v>
       </c>
-      <c r="P44" s="73"/>
-      <c r="Q44" s="72">
+      <c r="P44" s="68"/>
+      <c r="Q44" s="67">
         <f>Q43/20</f>
         <v>39.76876</v>
       </c>

</xml_diff>

<commit_message>
BOM changes after schematic redesign
</commit_message>
<xml_diff>
--- a/Deliverables/SM_Bottom Board/_BOM/eSpark BOM _Bottom (20 Boards).xlsx
+++ b/Deliverables/SM_Bottom Board/_BOM/eSpark BOM _Bottom (20 Boards).xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="236">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="234">
   <si>
     <t>Component list</t>
   </si>
@@ -67,9 +67,6 @@
     <t>C1</t>
   </si>
   <si>
-    <t>C2, C3, C4, C5, C6, C7, C8, C9, C10, C11, C15, C20, C32, C33, C34, C35, C36, C37, C50</t>
-  </si>
-  <si>
     <t>C12</t>
   </si>
   <si>
@@ -82,9 +79,6 @@
     <t>C18, C19</t>
   </si>
   <si>
-    <t>C31</t>
-  </si>
-  <si>
     <t>CF1</t>
   </si>
   <si>
@@ -121,9 +115,6 @@
     <t>R4, R5</t>
   </si>
   <si>
-    <t>R6</t>
-  </si>
-  <si>
     <t>R7, R8</t>
   </si>
   <si>
@@ -181,9 +172,6 @@
     <t>CAP CER 10PF 25V C0G 0201</t>
   </si>
   <si>
-    <t>CAP CER 10UF 25V X5R 0603</t>
-  </si>
-  <si>
     <t>Bidirectional 2.5V 3.5V 5V 20A (8/20us) DFN1006P2E TVS RoHS</t>
   </si>
   <si>
@@ -352,9 +340,6 @@
     <t>CGA1A2C0G1E100D030BA</t>
   </si>
   <si>
-    <t>CL10A106MA8NRNC</t>
-  </si>
-  <si>
     <t>ESD9L5.0ST5G</t>
   </si>
   <si>
@@ -493,9 +478,6 @@
     <t>10pF</t>
   </si>
   <si>
-    <t>10uF</t>
-  </si>
-  <si>
     <t>0R</t>
   </si>
   <si>
@@ -604,9 +586,6 @@
     <t>C7174</t>
   </si>
   <si>
-    <t>Low cost alternate. Design change needed due to different package size of capacitor</t>
-  </si>
-  <si>
     <t>C86017</t>
   </si>
   <si>
@@ -619,18 +598,12 @@
     <t>C2168858</t>
   </si>
   <si>
-    <t>C96446</t>
-  </si>
-  <si>
     <t>PESD2CAN,215</t>
   </si>
   <si>
     <t>C75176</t>
   </si>
   <si>
-    <t>Quantity changed from 2/board to 1/board due to 2xdiodes in single package. Design change required</t>
-  </si>
-  <si>
     <t>C82326</t>
   </si>
   <si>
@@ -697,9 +670,6 @@
     <t>C28730</t>
   </si>
   <si>
-    <t>Design change required. Only symbol change. No PCB or Footprint will change</t>
-  </si>
-  <si>
     <t>SN65HVDA1040AQDRQ1</t>
   </si>
   <si>
@@ -712,9 +682,6 @@
     <t>C123083</t>
   </si>
   <si>
-    <t>Design change required. Need approval from client first as this change will lead to firmware changes as well</t>
-  </si>
-  <si>
     <t>UTSource</t>
   </si>
   <si>
@@ -733,10 +700,49 @@
     <t>Cost per Board</t>
   </si>
   <si>
-    <t>Design change required.</t>
-  </si>
-  <si>
     <t>D1</t>
+  </si>
+  <si>
+    <t>C2, C3, C4, C5, C6, C7, C8, C9, C10, C11, C15, C32, C33, C34, C35, C36, C37, C50</t>
+  </si>
+  <si>
+    <t>Rx1, Rx2</t>
+  </si>
+  <si>
+    <t>RC0603FR-07100RL</t>
+  </si>
+  <si>
+    <t>100R</t>
+  </si>
+  <si>
+    <t>Quantity changed from 19/board to 18/board due to Encoder IC change</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">R6, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FFC00000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Rx3</t>
+    </r>
+  </si>
+  <si>
+    <t>Quantity changed from 1/board to 2/board due to Encoder IC change</t>
+  </si>
+  <si>
+    <t>RES SMD 100 OHM 1% 1/10W 0603</t>
+  </si>
+  <si>
+    <t>Added due to Encoder IC</t>
+  </si>
+  <si>
+    <t>C105588</t>
   </si>
 </sst>
 </file>
@@ -916,7 +922,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -953,6 +959,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="21">
     <border>
@@ -1191,7 +1209,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="85">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
@@ -1378,6 +1396,15 @@
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1387,13 +1414,34 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1440,7 +1488,7 @@
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1754,6 +1802,7 @@
     <col min="13" max="13" width="20.85546875" customWidth="1"/>
     <col min="14" max="15" width="19.140625" customWidth="1"/>
     <col min="16" max="18" width="29.42578125" customWidth="1"/>
+    <col min="20" max="20" width="18.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1767,14 +1816,14 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="69"/>
-      <c r="L1" s="69"/>
-      <c r="M1" s="69"/>
-      <c r="N1" s="69"/>
-      <c r="O1" s="69"/>
-      <c r="P1" s="69"/>
-      <c r="Q1" s="69"/>
-      <c r="R1" s="69"/>
+      <c r="K1" s="72"/>
+      <c r="L1" s="72"/>
+      <c r="M1" s="72"/>
+      <c r="N1" s="72"/>
+      <c r="O1" s="72"/>
+      <c r="P1" s="72"/>
+      <c r="Q1" s="72"/>
+      <c r="R1" s="72"/>
     </row>
     <row r="2" spans="1:18" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -1822,7 +1871,7 @@
       <c r="O3" s="4"/>
       <c r="P3" s="4"/>
       <c r="Q3" s="4"/>
-      <c r="R3" s="70"/>
+      <c r="R3" s="73"/>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -1846,7 +1895,7 @@
       <c r="O4" s="6"/>
       <c r="P4" s="6"/>
       <c r="Q4" s="59"/>
-      <c r="R4" s="71"/>
+      <c r="R4" s="74"/>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -1870,7 +1919,7 @@
       <c r="O5" s="5"/>
       <c r="P5" s="5"/>
       <c r="Q5" s="59"/>
-      <c r="R5" s="71"/>
+      <c r="R5" s="74"/>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -1890,7 +1939,7 @@
       <c r="O6" s="5"/>
       <c r="P6" s="5"/>
       <c r="Q6" s="59"/>
-      <c r="R6" s="71"/>
+      <c r="R6" s="74"/>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -1910,7 +1959,7 @@
       <c r="O7" s="7"/>
       <c r="P7" s="7"/>
       <c r="Q7" s="7"/>
-      <c r="R7" s="71"/>
+      <c r="R7" s="74"/>
     </row>
     <row r="8" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -1930,7 +1979,7 @@
       <c r="O8" s="7"/>
       <c r="P8" s="7"/>
       <c r="Q8" s="7"/>
-      <c r="R8" s="71"/>
+      <c r="R8" s="74"/>
     </row>
     <row r="9" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -1938,52 +1987,52 @@
         <v>4</v>
       </c>
       <c r="C9" s="29" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="D9" s="29" t="s">
         <v>10</v>
       </c>
       <c r="E9" s="30" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="F9" s="29" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="G9" s="30" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="H9" s="29" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="I9" s="29" t="s">
+        <v>171</v>
+      </c>
+      <c r="J9" s="29" t="s">
+        <v>172</v>
+      </c>
+      <c r="K9" s="30" t="s">
+        <v>142</v>
+      </c>
+      <c r="L9" s="29" t="s">
+        <v>156</v>
+      </c>
+      <c r="M9" s="29" t="s">
+        <v>173</v>
+      </c>
+      <c r="N9" s="29" t="s">
+        <v>174</v>
+      </c>
+      <c r="O9" s="29" t="s">
+        <v>175</v>
+      </c>
+      <c r="P9" s="29" t="s">
+        <v>176</v>
+      </c>
+      <c r="Q9" s="31" t="s">
         <v>177</v>
       </c>
-      <c r="J9" s="29" t="s">
+      <c r="R9" s="31" t="s">
         <v>178</v>
-      </c>
-      <c r="K9" s="30" t="s">
-        <v>147</v>
-      </c>
-      <c r="L9" s="29" t="s">
-        <v>162</v>
-      </c>
-      <c r="M9" s="29" t="s">
-        <v>179</v>
-      </c>
-      <c r="N9" s="29" t="s">
-        <v>180</v>
-      </c>
-      <c r="O9" s="29" t="s">
-        <v>181</v>
-      </c>
-      <c r="P9" s="29" t="s">
-        <v>182</v>
-      </c>
-      <c r="Q9" s="31" t="s">
-        <v>183</v>
-      </c>
-      <c r="R9" s="31" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="10" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1993,31 +2042,31 @@
         <v>1</v>
       </c>
       <c r="C10" s="37" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="D10" s="37" t="s">
         <v>11</v>
       </c>
       <c r="E10" s="38" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="F10" s="37" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="G10" s="38" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="H10" s="37" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="I10" s="37" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="J10" s="37" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="K10" s="38" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="L10" s="37">
         <v>1</v>
@@ -2030,7 +2079,7 @@
         <v>40</v>
       </c>
       <c r="O10" s="60" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="P10" s="37">
         <v>1.9199999999999998E-2</v>
@@ -2048,44 +2097,44 @@
         <v>2</v>
       </c>
       <c r="C11" s="39" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="D11" s="39" t="s">
-        <v>12</v>
+        <v>224</v>
       </c>
       <c r="E11" s="40" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="F11" s="39" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="G11" s="40" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="H11" s="39" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="I11" s="39" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="J11" s="39" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="K11" s="40" t="s">
-        <v>149</v>
-      </c>
-      <c r="L11" s="39">
-        <v>19</v>
+        <v>144</v>
+      </c>
+      <c r="L11" s="76">
+        <v>18</v>
       </c>
       <c r="M11" s="39">
         <f>L11*20</f>
-        <v>380</v>
+        <v>360</v>
       </c>
       <c r="N11" s="39">
         <v>400</v>
       </c>
       <c r="O11" s="61" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="P11" s="39">
         <v>1.4E-3</v>
@@ -2094,53 +2143,55 @@
         <f t="shared" ref="Q11:Q42" si="1">P11*N11</f>
         <v>0.55999999999999994</v>
       </c>
-      <c r="R11" s="42"/>
-    </row>
-    <row r="12" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R11" s="79" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
       <c r="B12" s="53">
         <f>ROW(B12) - ROW($B$9)</f>
         <v>3</v>
       </c>
       <c r="C12" s="37" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="D12" s="37" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E12" s="38" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="F12" s="37" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="G12" s="38" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="H12" s="37" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="I12" s="37" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="J12" s="37" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="K12" s="38" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="L12" s="37">
         <v>1</v>
       </c>
       <c r="M12" s="37">
-        <f t="shared" ref="M12:M42" si="2">L12*20</f>
+        <f t="shared" ref="M12:M31" si="2">L12*20</f>
         <v>20</v>
       </c>
       <c r="N12" s="37">
         <v>25</v>
       </c>
       <c r="O12" s="60" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="P12" s="37">
         <v>6.1499999999999999E-2</v>
@@ -2149,9 +2200,7 @@
         <f t="shared" si="1"/>
         <v>1.5375000000000001</v>
       </c>
-      <c r="R12" s="72" t="s">
-        <v>191</v>
-      </c>
+      <c r="R12" s="69"/>
     </row>
     <row r="13" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
@@ -2160,31 +2209,31 @@
         <v>4</v>
       </c>
       <c r="C13" s="39" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="D13" s="39" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E13" s="40" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="F13" s="39" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="G13" s="40" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="H13" s="39" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="I13" s="39" t="s">
+        <v>179</v>
+      </c>
+      <c r="J13" s="39" t="s">
         <v>185</v>
       </c>
-      <c r="J13" s="39" t="s">
-        <v>192</v>
-      </c>
       <c r="K13" s="40" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="L13" s="39">
         <v>2</v>
@@ -2197,7 +2246,7 @@
         <v>50</v>
       </c>
       <c r="O13" s="61" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="P13" s="39">
         <v>5.0099999999999999E-2</v>
@@ -2215,31 +2264,31 @@
         <v>5</v>
       </c>
       <c r="C14" s="37" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="D14" s="37" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E14" s="38" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="F14" s="37" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="G14" s="38" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="H14" s="37" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="I14" s="37" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="J14" s="37" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="K14" s="38" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="L14" s="37">
         <v>2</v>
@@ -2252,7 +2301,7 @@
         <v>100</v>
       </c>
       <c r="O14" s="60" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="P14" s="37">
         <v>3.3999999999999998E-3</v>
@@ -2270,31 +2319,31 @@
         <v>6</v>
       </c>
       <c r="C15" s="39" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="D15" s="39" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E15" s="40" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="F15" s="39" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="G15" s="40" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="H15" s="39" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="I15" s="39" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="J15" s="39" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="K15" s="40" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="L15" s="39">
         <v>2</v>
@@ -2307,7 +2356,7 @@
         <v>50</v>
       </c>
       <c r="O15" s="61" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="P15" s="39">
         <v>7.3000000000000001E-3</v>
@@ -2318,887 +2367,888 @@
       </c>
       <c r="R15" s="42"/>
     </row>
-    <row r="16" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:18" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
       <c r="B16" s="53">
-        <f>ROW(B16) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="C16" s="37" t="s">
-        <v>163</v>
-      </c>
-      <c r="D16" s="37" t="s">
-        <v>17</v>
-      </c>
-      <c r="E16" s="38" t="s">
-        <v>50</v>
-      </c>
-      <c r="F16" s="37" t="s">
-        <v>77</v>
-      </c>
-      <c r="G16" s="38" t="s">
-        <v>107</v>
-      </c>
-      <c r="H16" s="37" t="s">
-        <v>126</v>
-      </c>
-      <c r="I16" s="37" t="s">
-        <v>185</v>
-      </c>
-      <c r="J16" s="37" t="s">
-        <v>196</v>
-      </c>
-      <c r="K16" s="38" t="s">
-        <v>154</v>
-      </c>
-      <c r="L16" s="37">
+      <c r="C16" s="39" t="s">
+        <v>157</v>
+      </c>
+      <c r="D16" s="39" t="s">
+        <v>16</v>
+      </c>
+      <c r="E16" s="40" t="s">
+        <v>42</v>
+      </c>
+      <c r="F16" s="39" t="s">
+        <v>75</v>
+      </c>
+      <c r="G16" s="40" t="s">
+        <v>99</v>
+      </c>
+      <c r="H16" s="39" t="s">
+        <v>121</v>
+      </c>
+      <c r="I16" s="39" t="s">
+        <v>179</v>
+      </c>
+      <c r="J16" s="39" t="s">
+        <v>182</v>
+      </c>
+      <c r="K16" s="40" t="s">
+        <v>144</v>
+      </c>
+      <c r="L16" s="39">
         <v>1</v>
       </c>
-      <c r="M16" s="37">
+      <c r="M16" s="39">
         <f t="shared" si="2"/>
         <v>20</v>
       </c>
-      <c r="N16" s="37">
-        <v>40</v>
-      </c>
-      <c r="O16" s="60" t="s">
-        <v>187</v>
-      </c>
-      <c r="P16" s="37">
-        <v>1.49E-2</v>
-      </c>
-      <c r="Q16" s="41">
+      <c r="N16" s="39">
+        <v>100</v>
+      </c>
+      <c r="O16" s="61" t="s">
+        <v>181</v>
+      </c>
+      <c r="P16" s="39">
+        <v>1.4E-3</v>
+      </c>
+      <c r="Q16" s="42">
         <f t="shared" si="1"/>
-        <v>0.59599999999999997</v>
-      </c>
-      <c r="R16" s="41"/>
+        <v>0.13999999999999999</v>
+      </c>
+      <c r="R16" s="42"/>
     </row>
     <row r="17" spans="1:18" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
       <c r="B17" s="53">
-        <f t="shared" si="0"/>
+        <f>ROW(B17) - ROW($B$9)</f>
         <v>8</v>
       </c>
-      <c r="C17" s="39" t="s">
-        <v>163</v>
-      </c>
-      <c r="D17" s="39" t="s">
-        <v>18</v>
-      </c>
-      <c r="E17" s="40" t="s">
-        <v>45</v>
-      </c>
-      <c r="F17" s="39" t="s">
-        <v>79</v>
-      </c>
-      <c r="G17" s="40" t="s">
-        <v>103</v>
-      </c>
-      <c r="H17" s="39" t="s">
+      <c r="C17" s="37" t="s">
+        <v>158</v>
+      </c>
+      <c r="D17" s="37" t="s">
+        <v>223</v>
+      </c>
+      <c r="E17" s="38" t="s">
+        <v>47</v>
+      </c>
+      <c r="F17" s="37" t="s">
+        <v>168</v>
+      </c>
+      <c r="G17" s="37" t="s">
+        <v>77</v>
+      </c>
+      <c r="H17" s="37" t="s">
         <v>126</v>
       </c>
-      <c r="I17" s="39" t="s">
-        <v>185</v>
-      </c>
-      <c r="J17" s="39" t="s">
-        <v>188</v>
-      </c>
-      <c r="K17" s="40" t="s">
-        <v>149</v>
-      </c>
-      <c r="L17" s="39">
+      <c r="I17" s="37" t="s">
+        <v>189</v>
+      </c>
+      <c r="J17" s="37" t="s">
+        <v>190</v>
+      </c>
+      <c r="K17" s="38" t="s">
+        <v>179</v>
+      </c>
+      <c r="L17" s="70">
         <v>1</v>
       </c>
-      <c r="M17" s="39">
+      <c r="M17" s="37">
         <f t="shared" si="2"/>
         <v>20</v>
       </c>
-      <c r="N17" s="39">
-        <v>100</v>
-      </c>
-      <c r="O17" s="61" t="s">
-        <v>187</v>
-      </c>
-      <c r="P17" s="39">
-        <v>1.4E-3</v>
-      </c>
-      <c r="Q17" s="42">
+      <c r="N17" s="37">
+        <v>25</v>
+      </c>
+      <c r="O17" s="60" t="s">
+        <v>181</v>
+      </c>
+      <c r="P17" s="37">
+        <v>0.17119999999999999</v>
+      </c>
+      <c r="Q17" s="41">
         <f t="shared" si="1"/>
-        <v>0.13999999999999999</v>
-      </c>
-      <c r="R17" s="42"/>
-    </row>
-    <row r="18" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>4.2799999999999994</v>
+      </c>
+      <c r="R17" s="69"/>
+    </row>
+    <row r="18" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
       <c r="B18" s="53">
-        <f>ROW(B18) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="C18" s="37" t="s">
-        <v>164</v>
-      </c>
-      <c r="D18" s="37" t="s">
-        <v>235</v>
-      </c>
-      <c r="E18" s="38" t="s">
-        <v>51</v>
-      </c>
-      <c r="F18" s="37" t="s">
-        <v>174</v>
-      </c>
-      <c r="G18" s="37" t="s">
-        <v>81</v>
-      </c>
-      <c r="H18" s="37" t="s">
-        <v>131</v>
-      </c>
-      <c r="I18" s="37" t="s">
-        <v>197</v>
-      </c>
-      <c r="J18" s="37" t="s">
-        <v>198</v>
-      </c>
-      <c r="K18" s="38" t="s">
-        <v>185</v>
-      </c>
-      <c r="L18" s="73">
+      <c r="C18" s="39" t="s">
+        <v>158</v>
+      </c>
+      <c r="D18" s="39" t="s">
+        <v>17</v>
+      </c>
+      <c r="E18" s="40" t="s">
+        <v>48</v>
+      </c>
+      <c r="F18" s="39" t="s">
+        <v>78</v>
+      </c>
+      <c r="G18" s="40" t="s">
+        <v>103</v>
+      </c>
+      <c r="H18" s="39" t="s">
+        <v>127</v>
+      </c>
+      <c r="I18" s="39" t="s">
+        <v>179</v>
+      </c>
+      <c r="J18" s="39" t="s">
+        <v>191</v>
+      </c>
+      <c r="K18" s="40" t="s">
+        <v>179</v>
+      </c>
+      <c r="L18" s="39">
         <v>1</v>
       </c>
-      <c r="M18" s="37">
+      <c r="M18" s="39">
         <f t="shared" si="2"/>
         <v>20</v>
       </c>
-      <c r="N18" s="37">
+      <c r="N18" s="39">
         <v>25</v>
       </c>
-      <c r="O18" s="60" t="s">
-        <v>187</v>
-      </c>
-      <c r="P18" s="37">
-        <v>0.17119999999999999</v>
-      </c>
-      <c r="Q18" s="41">
+      <c r="O18" s="61" t="s">
+        <v>181</v>
+      </c>
+      <c r="P18" s="39">
+        <v>0.1066</v>
+      </c>
+      <c r="Q18" s="42">
         <f t="shared" si="1"/>
-        <v>4.2799999999999994</v>
-      </c>
-      <c r="R18" s="72" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="19" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>2.665</v>
+      </c>
+      <c r="R18" s="42"/>
+    </row>
+    <row r="19" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
       <c r="B19" s="53">
+        <f>ROW(B19) - ROW($B$9)</f>
+        <v>10</v>
+      </c>
+      <c r="C19" s="37" t="s">
+        <v>159</v>
+      </c>
+      <c r="D19" s="37" t="s">
+        <v>18</v>
+      </c>
+      <c r="E19" s="38" t="s">
+        <v>49</v>
+      </c>
+      <c r="F19" s="37" t="s">
+        <v>192</v>
+      </c>
+      <c r="G19" s="38" t="s">
+        <v>79</v>
+      </c>
+      <c r="H19" s="37" t="s">
+        <v>125</v>
+      </c>
+      <c r="I19" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="J19" s="37" t="s">
+        <v>193</v>
+      </c>
+      <c r="K19" s="38" t="s">
+        <v>179</v>
+      </c>
+      <c r="L19" s="37">
+        <v>4</v>
+      </c>
+      <c r="M19" s="37">
+        <f t="shared" si="2"/>
+        <v>80</v>
+      </c>
+      <c r="N19" s="37">
+        <v>100</v>
+      </c>
+      <c r="O19" s="60" t="s">
+        <v>181</v>
+      </c>
+      <c r="P19" s="37">
+        <v>2.9499999999999998E-2</v>
+      </c>
+      <c r="Q19" s="41">
+        <f t="shared" si="1"/>
+        <v>2.9499999999999997</v>
+      </c>
+      <c r="R19" s="41"/>
+    </row>
+    <row r="20" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="1"/>
+      <c r="B20" s="53">
         <f t="shared" si="0"/>
-        <v>10</v>
-      </c>
-      <c r="C19" s="39" t="s">
-        <v>164</v>
-      </c>
-      <c r="D19" s="39" t="s">
+        <v>11</v>
+      </c>
+      <c r="C20" s="39" t="s">
+        <v>160</v>
+      </c>
+      <c r="D20" s="39" t="s">
         <v>19</v>
       </c>
-      <c r="E19" s="40" t="s">
-        <v>52</v>
-      </c>
-      <c r="F19" s="39" t="s">
-        <v>82</v>
-      </c>
-      <c r="G19" s="40" t="s">
-        <v>108</v>
-      </c>
-      <c r="H19" s="39" t="s">
-        <v>132</v>
-      </c>
-      <c r="I19" s="39" t="s">
-        <v>185</v>
-      </c>
-      <c r="J19" s="39" t="s">
-        <v>200</v>
-      </c>
-      <c r="K19" s="40" t="s">
-        <v>185</v>
-      </c>
-      <c r="L19" s="39">
+      <c r="E20" s="40" t="s">
+        <v>50</v>
+      </c>
+      <c r="F20" s="39" t="s">
+        <v>168</v>
+      </c>
+      <c r="G20" s="40" t="s">
+        <v>80</v>
+      </c>
+      <c r="H20" s="39" t="s">
+        <v>128</v>
+      </c>
+      <c r="I20" s="39" t="s">
+        <v>179</v>
+      </c>
+      <c r="J20" s="39" t="s">
+        <v>179</v>
+      </c>
+      <c r="K20" s="40" t="s">
+        <v>179</v>
+      </c>
+      <c r="L20" s="39">
         <v>1</v>
       </c>
-      <c r="M19" s="39">
+      <c r="M20" s="39">
         <f t="shared" si="2"/>
         <v>20</v>
       </c>
-      <c r="N19" s="39">
+      <c r="N20" s="39">
         <v>25</v>
       </c>
-      <c r="O19" s="61" t="s">
-        <v>187</v>
-      </c>
-      <c r="P19" s="39">
-        <v>0.1066</v>
-      </c>
-      <c r="Q19" s="42">
+      <c r="O20" s="61" t="s">
+        <v>194</v>
+      </c>
+      <c r="P20" s="39">
+        <v>2.09</v>
+      </c>
+      <c r="Q20" s="42">
         <f t="shared" si="1"/>
-        <v>2.665</v>
-      </c>
-      <c r="R19" s="42"/>
-    </row>
-    <row r="20" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="1"/>
-      <c r="B20" s="53">
-        <f>ROW(B20) - ROW($B$9)</f>
-        <v>11</v>
-      </c>
-      <c r="C20" s="37" t="s">
-        <v>165</v>
-      </c>
-      <c r="D20" s="37" t="s">
-        <v>20</v>
-      </c>
-      <c r="E20" s="38" t="s">
-        <v>53</v>
-      </c>
-      <c r="F20" s="37" t="s">
-        <v>201</v>
-      </c>
-      <c r="G20" s="38" t="s">
-        <v>83</v>
-      </c>
-      <c r="H20" s="37" t="s">
-        <v>130</v>
-      </c>
-      <c r="I20" s="37" t="s">
-        <v>185</v>
-      </c>
-      <c r="J20" s="37" t="s">
-        <v>202</v>
-      </c>
-      <c r="K20" s="38" t="s">
-        <v>185</v>
-      </c>
-      <c r="L20" s="37">
-        <v>4</v>
-      </c>
-      <c r="M20" s="37">
-        <f t="shared" si="2"/>
-        <v>80</v>
-      </c>
-      <c r="N20" s="37">
-        <v>100</v>
-      </c>
-      <c r="O20" s="60" t="s">
-        <v>187</v>
-      </c>
-      <c r="P20" s="37">
-        <v>2.9499999999999998E-2</v>
-      </c>
-      <c r="Q20" s="41">
-        <f t="shared" si="1"/>
-        <v>2.9499999999999997</v>
-      </c>
-      <c r="R20" s="41"/>
-    </row>
-    <row r="21" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>52.25</v>
+      </c>
+      <c r="R20" s="42"/>
+    </row>
+    <row r="21" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1"/>
       <c r="B21" s="53">
-        <f t="shared" si="0"/>
+        <f>ROW(B21) - ROW($B$9)</f>
         <v>12</v>
       </c>
-      <c r="C21" s="39" t="s">
-        <v>166</v>
-      </c>
-      <c r="D21" s="39" t="s">
-        <v>21</v>
-      </c>
-      <c r="E21" s="40" t="s">
-        <v>54</v>
-      </c>
-      <c r="F21" s="39" t="s">
-        <v>174</v>
-      </c>
-      <c r="G21" s="40" t="s">
-        <v>84</v>
-      </c>
-      <c r="H21" s="39" t="s">
-        <v>133</v>
-      </c>
-      <c r="I21" s="39" t="s">
-        <v>185</v>
-      </c>
-      <c r="J21" s="39" t="s">
-        <v>185</v>
-      </c>
-      <c r="K21" s="40" t="s">
-        <v>185</v>
-      </c>
-      <c r="L21" s="39">
+      <c r="C21" s="37" t="s">
+        <v>159</v>
+      </c>
+      <c r="D21" s="37" t="s">
+        <v>20</v>
+      </c>
+      <c r="E21" s="38" t="s">
+        <v>51</v>
+      </c>
+      <c r="F21" s="37" t="s">
+        <v>81</v>
+      </c>
+      <c r="G21" s="38" t="s">
+        <v>104</v>
+      </c>
+      <c r="H21" s="37" t="s">
+        <v>129</v>
+      </c>
+      <c r="I21" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="J21" s="37" t="s">
+        <v>195</v>
+      </c>
+      <c r="K21" s="38" t="s">
+        <v>179</v>
+      </c>
+      <c r="L21" s="37">
         <v>1</v>
       </c>
-      <c r="M21" s="39">
+      <c r="M21" s="37">
         <f t="shared" si="2"/>
         <v>20</v>
       </c>
-      <c r="N21" s="39">
+      <c r="N21" s="37">
         <v>25</v>
       </c>
-      <c r="O21" s="61" t="s">
-        <v>203</v>
-      </c>
-      <c r="P21" s="39">
-        <v>2.09</v>
-      </c>
-      <c r="Q21" s="42">
+      <c r="O21" s="60" t="s">
+        <v>181</v>
+      </c>
+      <c r="P21" s="37">
+        <v>9.8500000000000004E-2</v>
+      </c>
+      <c r="Q21" s="41">
         <f t="shared" si="1"/>
-        <v>52.25</v>
-      </c>
-      <c r="R21" s="42"/>
-    </row>
-    <row r="22" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>2.4624999999999999</v>
+      </c>
+      <c r="R21" s="41"/>
+    </row>
+    <row r="22" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
       <c r="B22" s="53">
-        <f>ROW(B22) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="C22" s="37" t="s">
-        <v>165</v>
-      </c>
-      <c r="D22" s="37" t="s">
-        <v>22</v>
-      </c>
-      <c r="E22" s="38" t="s">
-        <v>55</v>
-      </c>
-      <c r="F22" s="37" t="s">
-        <v>85</v>
-      </c>
-      <c r="G22" s="38" t="s">
-        <v>109</v>
-      </c>
-      <c r="H22" s="37" t="s">
-        <v>134</v>
-      </c>
-      <c r="I22" s="37" t="s">
-        <v>185</v>
-      </c>
-      <c r="J22" s="37" t="s">
-        <v>204</v>
-      </c>
-      <c r="K22" s="38" t="s">
-        <v>185</v>
-      </c>
-      <c r="L22" s="37">
+      <c r="C22" s="39" t="s">
+        <v>161</v>
+      </c>
+      <c r="D22" s="39" t="s">
+        <v>21</v>
+      </c>
+      <c r="E22" s="40" t="s">
+        <v>52</v>
+      </c>
+      <c r="F22" s="39" t="s">
+        <v>82</v>
+      </c>
+      <c r="G22" s="40" t="s">
+        <v>105</v>
+      </c>
+      <c r="H22" s="39" t="s">
+        <v>130</v>
+      </c>
+      <c r="I22" s="39" t="s">
+        <v>196</v>
+      </c>
+      <c r="J22" s="39" t="s">
+        <v>197</v>
+      </c>
+      <c r="K22" s="40" t="s">
+        <v>179</v>
+      </c>
+      <c r="L22" s="39">
         <v>1</v>
       </c>
-      <c r="M22" s="37">
+      <c r="M22" s="39">
         <f t="shared" si="2"/>
         <v>20</v>
       </c>
-      <c r="N22" s="37">
-        <v>25</v>
-      </c>
-      <c r="O22" s="60" t="s">
-        <v>187</v>
-      </c>
-      <c r="P22" s="37">
-        <v>9.8500000000000004E-2</v>
-      </c>
-      <c r="Q22" s="41">
+      <c r="N22" s="39">
+        <v>30</v>
+      </c>
+      <c r="O22" s="61" t="s">
+        <v>181</v>
+      </c>
+      <c r="P22" s="39">
+        <v>4.2200000000000001E-2</v>
+      </c>
+      <c r="Q22" s="42">
         <f t="shared" si="1"/>
-        <v>2.4624999999999999</v>
-      </c>
-      <c r="R22" s="41"/>
+        <v>1.266</v>
+      </c>
+      <c r="R22" s="42"/>
     </row>
     <row r="23" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1"/>
       <c r="B23" s="53">
-        <f t="shared" si="0"/>
+        <f>ROW(B23) - ROW($B$9)</f>
         <v>14</v>
       </c>
-      <c r="C23" s="39" t="s">
-        <v>167</v>
-      </c>
-      <c r="D23" s="39" t="s">
-        <v>23</v>
-      </c>
-      <c r="E23" s="40" t="s">
-        <v>56</v>
-      </c>
-      <c r="F23" s="39" t="s">
-        <v>86</v>
-      </c>
-      <c r="G23" s="40" t="s">
-        <v>110</v>
-      </c>
-      <c r="H23" s="39" t="s">
-        <v>135</v>
-      </c>
-      <c r="I23" s="39" t="s">
-        <v>205</v>
-      </c>
-      <c r="J23" s="39" t="s">
-        <v>206</v>
-      </c>
-      <c r="K23" s="40" t="s">
-        <v>185</v>
-      </c>
-      <c r="L23" s="39">
+      <c r="C23" s="37" t="s">
+        <v>162</v>
+      </c>
+      <c r="D23" s="37" t="s">
+        <v>22</v>
+      </c>
+      <c r="E23" s="38" t="s">
+        <v>53</v>
+      </c>
+      <c r="F23" s="37" t="s">
+        <v>168</v>
+      </c>
+      <c r="G23" s="38" t="s">
+        <v>83</v>
+      </c>
+      <c r="H23" s="37" t="s">
+        <v>131</v>
+      </c>
+      <c r="I23" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="J23" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="K23" s="38" t="s">
+        <v>179</v>
+      </c>
+      <c r="L23" s="37">
         <v>1</v>
       </c>
-      <c r="M23" s="39">
+      <c r="M23" s="37">
         <f t="shared" si="2"/>
         <v>20</v>
       </c>
-      <c r="N23" s="39">
-        <v>30</v>
-      </c>
-      <c r="O23" s="61" t="s">
-        <v>187</v>
-      </c>
-      <c r="P23" s="39">
-        <v>4.2200000000000001E-2</v>
-      </c>
-      <c r="Q23" s="42">
+      <c r="N23" s="37">
+        <v>25</v>
+      </c>
+      <c r="O23" s="60" t="s">
+        <v>198</v>
+      </c>
+      <c r="P23" s="37">
+        <v>0.30840000000000001</v>
+      </c>
+      <c r="Q23" s="41">
         <f t="shared" si="1"/>
-        <v>1.266</v>
-      </c>
-      <c r="R23" s="42"/>
+        <v>7.71</v>
+      </c>
+      <c r="R23" s="41"/>
     </row>
     <row r="24" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1"/>
       <c r="B24" s="53">
-        <f>ROW(B24) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="C24" s="37" t="s">
-        <v>168</v>
-      </c>
-      <c r="D24" s="37" t="s">
+      <c r="C24" s="39" t="s">
+        <v>163</v>
+      </c>
+      <c r="D24" s="39" t="s">
+        <v>23</v>
+      </c>
+      <c r="E24" s="40" t="s">
+        <v>54</v>
+      </c>
+      <c r="F24" s="39" t="s">
+        <v>84</v>
+      </c>
+      <c r="G24" s="40" t="s">
+        <v>106</v>
+      </c>
+      <c r="H24" s="39" t="s">
+        <v>132</v>
+      </c>
+      <c r="I24" s="39" t="s">
+        <v>179</v>
+      </c>
+      <c r="J24" s="39" t="s">
+        <v>199</v>
+      </c>
+      <c r="K24" s="40" t="s">
+        <v>179</v>
+      </c>
+      <c r="L24" s="39">
+        <v>2</v>
+      </c>
+      <c r="M24" s="39">
+        <f t="shared" si="2"/>
+        <v>40</v>
+      </c>
+      <c r="N24" s="39">
+        <v>60</v>
+      </c>
+      <c r="O24" s="61" t="s">
+        <v>181</v>
+      </c>
+      <c r="P24" s="39">
+        <v>3.4799999999999998E-2</v>
+      </c>
+      <c r="Q24" s="42">
+        <f t="shared" si="1"/>
+        <v>2.0880000000000001</v>
+      </c>
+      <c r="R24" s="42"/>
+    </row>
+    <row r="25" spans="1:18" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="1"/>
+      <c r="B25" s="53">
+        <f>ROW(B25) - ROW($B$9)</f>
+        <v>16</v>
+      </c>
+      <c r="C25" s="37" t="s">
+        <v>164</v>
+      </c>
+      <c r="D25" s="37" t="s">
         <v>24</v>
       </c>
-      <c r="E24" s="38" t="s">
+      <c r="E25" s="38" t="s">
+        <v>55</v>
+      </c>
+      <c r="F25" s="37" t="s">
+        <v>85</v>
+      </c>
+      <c r="G25" s="38" t="s">
+        <v>107</v>
+      </c>
+      <c r="H25" s="37" t="s">
+        <v>124</v>
+      </c>
+      <c r="I25" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="J25" s="37" t="s">
+        <v>200</v>
+      </c>
+      <c r="K25" s="38" t="s">
+        <v>149</v>
+      </c>
+      <c r="L25" s="37">
+        <v>40</v>
+      </c>
+      <c r="M25" s="37">
+        <f t="shared" si="2"/>
+        <v>800</v>
+      </c>
+      <c r="N25" s="37">
+        <v>900</v>
+      </c>
+      <c r="O25" s="60" t="s">
+        <v>181</v>
+      </c>
+      <c r="P25" s="37">
+        <v>8.9999999999999998E-4</v>
+      </c>
+      <c r="Q25" s="41">
+        <f t="shared" si="1"/>
+        <v>0.80999999999999994</v>
+      </c>
+      <c r="R25" s="41"/>
+    </row>
+    <row r="26" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="1"/>
+      <c r="B26" s="53">
+        <f t="shared" si="0"/>
+        <v>17</v>
+      </c>
+      <c r="C26" s="39" t="s">
+        <v>164</v>
+      </c>
+      <c r="D26" s="39" t="s">
+        <v>25</v>
+      </c>
+      <c r="E26" s="40" t="s">
+        <v>56</v>
+      </c>
+      <c r="F26" s="39" t="s">
+        <v>86</v>
+      </c>
+      <c r="G26" s="40" t="s">
+        <v>108</v>
+      </c>
+      <c r="H26" s="39" t="s">
+        <v>124</v>
+      </c>
+      <c r="I26" s="39" t="s">
+        <v>179</v>
+      </c>
+      <c r="J26" s="39" t="s">
+        <v>201</v>
+      </c>
+      <c r="K26" s="40" t="s">
+        <v>150</v>
+      </c>
+      <c r="L26" s="39">
+        <v>7</v>
+      </c>
+      <c r="M26" s="39">
+        <f t="shared" si="2"/>
+        <v>140</v>
+      </c>
+      <c r="N26" s="39">
+        <v>200</v>
+      </c>
+      <c r="O26" s="61" t="s">
+        <v>181</v>
+      </c>
+      <c r="P26" s="39">
+        <v>1.1999999999999999E-3</v>
+      </c>
+      <c r="Q26" s="42">
+        <f t="shared" si="1"/>
+        <v>0.24</v>
+      </c>
+      <c r="R26" s="42"/>
+    </row>
+    <row r="27" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="1"/>
+      <c r="B27" s="53">
+        <f>ROW(B27) - ROW($B$9)</f>
+        <v>18</v>
+      </c>
+      <c r="C27" s="37" t="s">
+        <v>164</v>
+      </c>
+      <c r="D27" s="37" t="s">
+        <v>26</v>
+      </c>
+      <c r="E27" s="38" t="s">
         <v>57</v>
       </c>
-      <c r="F24" s="37" t="s">
-        <v>174</v>
-      </c>
-      <c r="G24" s="38" t="s">
-        <v>87</v>
-      </c>
-      <c r="H24" s="37" t="s">
-        <v>136</v>
-      </c>
-      <c r="I24" s="37" t="s">
-        <v>185</v>
-      </c>
-      <c r="J24" s="37" t="s">
-        <v>185</v>
-      </c>
-      <c r="K24" s="38" t="s">
-        <v>185</v>
-      </c>
-      <c r="L24" s="37">
+      <c r="F27" s="37" t="s">
+        <v>85</v>
+      </c>
+      <c r="G27" s="38" t="s">
+        <v>109</v>
+      </c>
+      <c r="H27" s="37" t="s">
+        <v>133</v>
+      </c>
+      <c r="I27" s="37" t="s">
+        <v>202</v>
+      </c>
+      <c r="J27" s="37" t="s">
+        <v>203</v>
+      </c>
+      <c r="K27" s="38" t="s">
+        <v>151</v>
+      </c>
+      <c r="L27" s="37">
         <v>1</v>
       </c>
-      <c r="M24" s="37">
+      <c r="M27" s="37">
         <f t="shared" si="2"/>
         <v>20</v>
       </c>
-      <c r="N24" s="37">
-        <v>25</v>
-      </c>
-      <c r="O24" s="60" t="s">
-        <v>207</v>
-      </c>
-      <c r="P24" s="37">
-        <v>0.30840000000000001</v>
-      </c>
-      <c r="Q24" s="41">
+      <c r="N27" s="37">
+        <v>100</v>
+      </c>
+      <c r="O27" s="60" t="s">
+        <v>181</v>
+      </c>
+      <c r="P27" s="37">
+        <v>2.0999999999999999E-3</v>
+      </c>
+      <c r="Q27" s="41">
         <f t="shared" si="1"/>
-        <v>7.71</v>
-      </c>
-      <c r="R24" s="41"/>
-    </row>
-    <row r="25" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="1"/>
-      <c r="B25" s="53">
+        <v>0.21</v>
+      </c>
+      <c r="R27" s="41"/>
+    </row>
+    <row r="28" spans="1:18" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="1"/>
+      <c r="B28" s="53">
         <f t="shared" si="0"/>
-        <v>16</v>
-      </c>
-      <c r="C25" s="39" t="s">
-        <v>169</v>
-      </c>
-      <c r="D25" s="39" t="s">
-        <v>25</v>
-      </c>
-      <c r="E25" s="40" t="s">
+        <v>19</v>
+      </c>
+      <c r="C28" s="39" t="s">
+        <v>164</v>
+      </c>
+      <c r="D28" s="39" t="s">
+        <v>27</v>
+      </c>
+      <c r="E28" s="40" t="s">
         <v>58</v>
       </c>
-      <c r="F25" s="39" t="s">
-        <v>88</v>
-      </c>
-      <c r="G25" s="40" t="s">
-        <v>111</v>
-      </c>
-      <c r="H25" s="39" t="s">
-        <v>137</v>
-      </c>
-      <c r="I25" s="39" t="s">
-        <v>185</v>
-      </c>
-      <c r="J25" s="39" t="s">
-        <v>208</v>
-      </c>
-      <c r="K25" s="40" t="s">
-        <v>185</v>
-      </c>
-      <c r="L25" s="39">
+      <c r="F28" s="39" t="s">
+        <v>86</v>
+      </c>
+      <c r="G28" s="40" t="s">
+        <v>110</v>
+      </c>
+      <c r="H28" s="39" t="s">
+        <v>124</v>
+      </c>
+      <c r="I28" s="39" t="s">
+        <v>179</v>
+      </c>
+      <c r="J28" s="39" t="s">
+        <v>204</v>
+      </c>
+      <c r="K28" s="40" t="s">
+        <v>152</v>
+      </c>
+      <c r="L28" s="39">
         <v>2</v>
       </c>
-      <c r="M25" s="39">
+      <c r="M28" s="39">
         <f t="shared" si="2"/>
         <v>40</v>
       </c>
-      <c r="N25" s="39">
-        <v>60</v>
-      </c>
-      <c r="O25" s="61" t="s">
-        <v>187</v>
-      </c>
-      <c r="P25" s="39">
-        <v>3.4799999999999998E-2</v>
-      </c>
-      <c r="Q25" s="42">
+      <c r="N28" s="39">
+        <v>100</v>
+      </c>
+      <c r="O28" s="61" t="s">
+        <v>181</v>
+      </c>
+      <c r="P28" s="39">
+        <v>1.4E-3</v>
+      </c>
+      <c r="Q28" s="42">
         <f t="shared" si="1"/>
-        <v>2.0880000000000001</v>
-      </c>
-      <c r="R25" s="42"/>
-    </row>
-    <row r="26" spans="1:18" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="1"/>
-      <c r="B26" s="53">
-        <f>ROW(B26) - ROW($B$9)</f>
-        <v>17</v>
-      </c>
-      <c r="C26" s="37" t="s">
-        <v>170</v>
-      </c>
-      <c r="D26" s="37" t="s">
-        <v>26</v>
-      </c>
-      <c r="E26" s="38" t="s">
-        <v>59</v>
-      </c>
-      <c r="F26" s="37" t="s">
-        <v>89</v>
-      </c>
-      <c r="G26" s="38" t="s">
-        <v>112</v>
-      </c>
-      <c r="H26" s="37" t="s">
-        <v>129</v>
-      </c>
-      <c r="I26" s="37" t="s">
-        <v>185</v>
-      </c>
-      <c r="J26" s="37" t="s">
-        <v>209</v>
-      </c>
-      <c r="K26" s="38" t="s">
-        <v>155</v>
-      </c>
-      <c r="L26" s="37">
-        <v>40</v>
-      </c>
-      <c r="M26" s="37">
-        <f t="shared" si="2"/>
-        <v>800</v>
-      </c>
-      <c r="N26" s="37">
-        <v>900</v>
-      </c>
-      <c r="O26" s="60" t="s">
-        <v>187</v>
-      </c>
-      <c r="P26" s="37">
-        <v>8.9999999999999998E-4</v>
-      </c>
-      <c r="Q26" s="41">
-        <f t="shared" si="1"/>
-        <v>0.80999999999999994</v>
-      </c>
-      <c r="R26" s="41"/>
-    </row>
-    <row r="27" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="1"/>
-      <c r="B27" s="53">
-        <f t="shared" si="0"/>
-        <v>18</v>
-      </c>
-      <c r="C27" s="39" t="s">
-        <v>170</v>
-      </c>
-      <c r="D27" s="39" t="s">
-        <v>27</v>
-      </c>
-      <c r="E27" s="40" t="s">
-        <v>60</v>
-      </c>
-      <c r="F27" s="39" t="s">
-        <v>90</v>
-      </c>
-      <c r="G27" s="40" t="s">
-        <v>113</v>
-      </c>
-      <c r="H27" s="39" t="s">
-        <v>129</v>
-      </c>
-      <c r="I27" s="39" t="s">
-        <v>185</v>
-      </c>
-      <c r="J27" s="39" t="s">
-        <v>210</v>
-      </c>
-      <c r="K27" s="40" t="s">
-        <v>156</v>
-      </c>
-      <c r="L27" s="39">
-        <v>7</v>
-      </c>
-      <c r="M27" s="39">
-        <f t="shared" si="2"/>
-        <v>140</v>
-      </c>
-      <c r="N27" s="39">
-        <v>200</v>
-      </c>
-      <c r="O27" s="61" t="s">
-        <v>187</v>
-      </c>
-      <c r="P27" s="39">
-        <v>1.1999999999999999E-3</v>
-      </c>
-      <c r="Q27" s="42">
-        <f t="shared" si="1"/>
-        <v>0.24</v>
-      </c>
-      <c r="R27" s="42"/>
-    </row>
-    <row r="28" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="1"/>
-      <c r="B28" s="53">
-        <f>ROW(B28) - ROW($B$9)</f>
-        <v>19</v>
-      </c>
-      <c r="C28" s="37" t="s">
-        <v>170</v>
-      </c>
-      <c r="D28" s="37" t="s">
-        <v>28</v>
-      </c>
-      <c r="E28" s="38" t="s">
-        <v>61</v>
-      </c>
-      <c r="F28" s="37" t="s">
-        <v>89</v>
-      </c>
-      <c r="G28" s="38" t="s">
-        <v>114</v>
-      </c>
-      <c r="H28" s="37" t="s">
-        <v>138</v>
-      </c>
-      <c r="I28" s="37" t="s">
-        <v>211</v>
-      </c>
-      <c r="J28" s="37" t="s">
-        <v>212</v>
-      </c>
-      <c r="K28" s="38" t="s">
-        <v>157</v>
-      </c>
-      <c r="L28" s="37">
-        <v>1</v>
-      </c>
-      <c r="M28" s="37">
-        <f t="shared" si="2"/>
-        <v>20</v>
-      </c>
-      <c r="N28" s="37">
-        <v>100</v>
-      </c>
-      <c r="O28" s="60" t="s">
-        <v>187</v>
-      </c>
-      <c r="P28" s="37">
-        <v>2.0999999999999999E-3</v>
-      </c>
-      <c r="Q28" s="41">
-        <f t="shared" si="1"/>
-        <v>0.21</v>
-      </c>
-      <c r="R28" s="41"/>
+        <v>0.13999999999999999</v>
+      </c>
+      <c r="R28" s="42"/>
     </row>
     <row r="29" spans="1:18" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1"/>
       <c r="B29" s="53">
-        <f t="shared" si="0"/>
+        <f>ROW(B29) - ROW($B$9)</f>
         <v>20</v>
       </c>
-      <c r="C29" s="39" t="s">
-        <v>170</v>
-      </c>
-      <c r="D29" s="39" t="s">
-        <v>29</v>
-      </c>
-      <c r="E29" s="40" t="s">
-        <v>62</v>
-      </c>
-      <c r="F29" s="39" t="s">
-        <v>90</v>
-      </c>
-      <c r="G29" s="40" t="s">
-        <v>115</v>
-      </c>
-      <c r="H29" s="39" t="s">
-        <v>129</v>
-      </c>
-      <c r="I29" s="39" t="s">
-        <v>185</v>
-      </c>
-      <c r="J29" s="39" t="s">
-        <v>213</v>
-      </c>
-      <c r="K29" s="40" t="s">
-        <v>158</v>
-      </c>
-      <c r="L29" s="39">
+      <c r="C29" s="37" t="s">
+        <v>164</v>
+      </c>
+      <c r="D29" s="77" t="s">
+        <v>229</v>
+      </c>
+      <c r="E29" s="38" t="s">
+        <v>59</v>
+      </c>
+      <c r="F29" s="37" t="s">
+        <v>86</v>
+      </c>
+      <c r="G29" s="38" t="s">
+        <v>111</v>
+      </c>
+      <c r="H29" s="37" t="s">
+        <v>124</v>
+      </c>
+      <c r="I29" s="37" t="s">
+        <v>179</v>
+      </c>
+      <c r="J29" s="37" t="s">
+        <v>205</v>
+      </c>
+      <c r="K29" s="38" t="s">
+        <v>153</v>
+      </c>
+      <c r="L29" s="78">
         <v>2</v>
       </c>
-      <c r="M29" s="39">
+      <c r="M29" s="37">
         <f t="shared" si="2"/>
         <v>40</v>
       </c>
-      <c r="N29" s="39">
+      <c r="N29" s="37">
         <v>100</v>
       </c>
-      <c r="O29" s="61" t="s">
-        <v>187</v>
-      </c>
-      <c r="P29" s="39">
+      <c r="O29" s="60" t="s">
+        <v>181</v>
+      </c>
+      <c r="P29" s="37">
         <v>1.4E-3</v>
       </c>
-      <c r="Q29" s="42">
+      <c r="Q29" s="41">
         <f t="shared" si="1"/>
         <v>0.13999999999999999</v>
       </c>
-      <c r="R29" s="42"/>
-    </row>
-    <row r="30" spans="1:18" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R29" s="69" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="30" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1"/>
       <c r="B30" s="53">
-        <f>ROW(B30) - ROW($B$9)</f>
+        <f t="shared" si="0"/>
         <v>21</v>
       </c>
-      <c r="C30" s="37" t="s">
-        <v>170</v>
-      </c>
-      <c r="D30" s="37" t="s">
-        <v>30</v>
-      </c>
-      <c r="E30" s="38" t="s">
-        <v>63</v>
-      </c>
-      <c r="F30" s="37" t="s">
-        <v>90</v>
-      </c>
-      <c r="G30" s="38" t="s">
-        <v>116</v>
-      </c>
-      <c r="H30" s="37" t="s">
-        <v>129</v>
-      </c>
-      <c r="I30" s="37" t="s">
-        <v>185</v>
-      </c>
-      <c r="J30" s="37" t="s">
-        <v>214</v>
-      </c>
-      <c r="K30" s="38" t="s">
-        <v>159</v>
-      </c>
-      <c r="L30" s="37">
-        <v>1</v>
-      </c>
-      <c r="M30" s="37">
+      <c r="C30" s="39" t="s">
+        <v>164</v>
+      </c>
+      <c r="D30" s="39" t="s">
+        <v>28</v>
+      </c>
+      <c r="E30" s="40" t="s">
+        <v>60</v>
+      </c>
+      <c r="F30" s="39" t="s">
+        <v>86</v>
+      </c>
+      <c r="G30" s="40" t="s">
+        <v>112</v>
+      </c>
+      <c r="H30" s="39" t="s">
+        <v>124</v>
+      </c>
+      <c r="I30" s="39" t="s">
+        <v>206</v>
+      </c>
+      <c r="J30" s="39" t="s">
+        <v>207</v>
+      </c>
+      <c r="K30" s="40" t="s">
+        <v>154</v>
+      </c>
+      <c r="L30" s="39">
+        <v>2</v>
+      </c>
+      <c r="M30" s="39">
         <f t="shared" si="2"/>
-        <v>20</v>
-      </c>
-      <c r="N30" s="37">
-        <v>100</v>
-      </c>
-      <c r="O30" s="60" t="s">
-        <v>187</v>
-      </c>
-      <c r="P30" s="37">
-        <v>1.4E-3</v>
-      </c>
-      <c r="Q30" s="41">
+        <v>40</v>
+      </c>
+      <c r="N30" s="39">
+        <v>50</v>
+      </c>
+      <c r="O30" s="61" t="s">
+        <v>181</v>
+      </c>
+      <c r="P30" s="39">
+        <v>1.01E-2</v>
+      </c>
+      <c r="Q30" s="42">
         <f t="shared" si="1"/>
-        <v>0.13999999999999999</v>
-      </c>
-      <c r="R30" s="41"/>
+        <v>0.505</v>
+      </c>
+      <c r="R30" s="42"/>
     </row>
     <row r="31" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="1"/>
       <c r="B31" s="53">
-        <f t="shared" si="0"/>
         <v>22</v>
       </c>
-      <c r="C31" s="39" t="s">
-        <v>170</v>
-      </c>
-      <c r="D31" s="39" t="s">
-        <v>31</v>
-      </c>
-      <c r="E31" s="40" t="s">
-        <v>64</v>
-      </c>
-      <c r="F31" s="39" t="s">
-        <v>90</v>
-      </c>
-      <c r="G31" s="40" t="s">
-        <v>117</v>
-      </c>
-      <c r="H31" s="39" t="s">
-        <v>129</v>
-      </c>
-      <c r="I31" s="39" t="s">
-        <v>215</v>
-      </c>
-      <c r="J31" s="39" t="s">
-        <v>216</v>
-      </c>
-      <c r="K31" s="40" t="s">
-        <v>160</v>
-      </c>
-      <c r="L31" s="39">
+      <c r="C31" s="80" t="s">
+        <v>164</v>
+      </c>
+      <c r="D31" s="75" t="s">
+        <v>225</v>
+      </c>
+      <c r="E31" s="81" t="s">
+        <v>231</v>
+      </c>
+      <c r="F31" s="75" t="s">
+        <v>86</v>
+      </c>
+      <c r="G31" s="81" t="s">
+        <v>226</v>
+      </c>
+      <c r="H31" s="75" t="s">
+        <v>124</v>
+      </c>
+      <c r="I31" s="80" t="s">
+        <v>179</v>
+      </c>
+      <c r="J31" s="80" t="s">
+        <v>233</v>
+      </c>
+      <c r="K31" s="81" t="s">
+        <v>227</v>
+      </c>
+      <c r="L31" s="75">
         <v>2</v>
       </c>
-      <c r="M31" s="39">
-        <f t="shared" si="2"/>
+      <c r="M31" s="75">
+        <f>L31*20</f>
         <v>40</v>
       </c>
-      <c r="N31" s="39">
-        <v>50</v>
-      </c>
-      <c r="O31" s="61" t="s">
-        <v>187</v>
-      </c>
-      <c r="P31" s="39">
-        <v>1.01E-2</v>
-      </c>
-      <c r="Q31" s="42">
-        <f t="shared" si="1"/>
-        <v>0.505</v>
-      </c>
-      <c r="R31" s="42"/>
+      <c r="N31" s="80">
+        <v>100</v>
+      </c>
+      <c r="O31" s="82" t="s">
+        <v>181</v>
+      </c>
+      <c r="P31" s="80">
+        <v>1E-3</v>
+      </c>
+      <c r="Q31" s="83">
+        <f>P31*N31</f>
+        <v>0.1</v>
+      </c>
+      <c r="R31" s="84" t="s">
+        <v>232</v>
+      </c>
     </row>
     <row r="32" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="1"/>
@@ -3207,44 +3257,44 @@
         <v>23</v>
       </c>
       <c r="C32" s="62" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="D32" s="62" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="E32" s="63" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="F32" s="62" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="G32" s="63" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="H32" s="62" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="I32" s="62" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="J32" s="62" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="K32" s="63" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="L32" s="62">
         <v>8</v>
       </c>
       <c r="M32" s="62">
-        <f t="shared" si="2"/>
+        <f>L32*20</f>
         <v>160</v>
       </c>
       <c r="N32" s="62">
         <v>160</v>
       </c>
       <c r="O32" s="62" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="P32" s="62">
         <v>0</v>
@@ -3254,7 +3304,7 @@
         <v>0</v>
       </c>
       <c r="R32" s="64" t="s">
-        <v>217</v>
+        <v>208</v>
       </c>
     </row>
     <row r="33" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3264,44 +3314,44 @@
         <v>24</v>
       </c>
       <c r="C33" s="39" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="D33" s="39" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="E33" s="40" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="F33" s="39" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="G33" s="40" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="H33" s="39" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="I33" s="39" t="s">
-        <v>218</v>
+        <v>209</v>
       </c>
       <c r="J33" s="39" t="s">
-        <v>219</v>
+        <v>210</v>
       </c>
       <c r="K33" s="40" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="L33" s="39">
         <v>1</v>
       </c>
       <c r="M33" s="39">
-        <f t="shared" si="2"/>
+        <f>L33*20</f>
         <v>20</v>
       </c>
       <c r="N33" s="39">
         <v>30</v>
       </c>
       <c r="O33" s="61" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="P33" s="39">
         <v>4.9599999999999998E-2</v>
@@ -3310,55 +3360,53 @@
         <f t="shared" si="1"/>
         <v>1.488</v>
       </c>
-      <c r="R33" s="74" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="34" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R33" s="71"/>
+    </row>
+    <row r="34" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="1"/>
       <c r="B34" s="53">
         <f>ROW(B34) - ROW($B$9)</f>
         <v>25</v>
       </c>
       <c r="C34" s="37" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="D34" s="37" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="E34" s="38" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="F34" s="37" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="G34" s="38" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="H34" s="37" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="I34" s="37" t="s">
-        <v>220</v>
+        <v>211</v>
       </c>
       <c r="J34" s="37" t="s">
-        <v>221</v>
+        <v>212</v>
       </c>
       <c r="K34" s="38" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="L34" s="37">
         <v>1</v>
       </c>
       <c r="M34" s="37">
-        <f t="shared" si="2"/>
+        <f>L34*20</f>
         <v>20</v>
       </c>
       <c r="N34" s="37">
         <v>22</v>
       </c>
       <c r="O34" s="60" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="P34" s="37">
         <v>10.947699999999999</v>
@@ -3367,55 +3415,53 @@
         <f t="shared" si="1"/>
         <v>240.84939999999997</v>
       </c>
-      <c r="R34" s="72" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="35" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R34" s="69"/>
+    </row>
+    <row r="35" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="1"/>
       <c r="B35" s="53">
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
       <c r="C35" s="39" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="D35" s="39" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E35" s="40" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="F35" s="39" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="G35" s="40" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="H35" s="39" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="I35" s="39" t="s">
-        <v>223</v>
+        <v>213</v>
       </c>
       <c r="J35" s="39" t="s">
-        <v>224</v>
+        <v>214</v>
       </c>
       <c r="K35" s="40" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="L35" s="39">
         <v>1</v>
       </c>
       <c r="M35" s="39">
-        <f t="shared" si="2"/>
+        <f>L35*20</f>
         <v>20</v>
       </c>
       <c r="N35" s="39">
         <v>22</v>
       </c>
       <c r="O35" s="61" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="P35" s="39">
         <v>3.0078999999999998</v>
@@ -3424,55 +3470,53 @@
         <f t="shared" si="1"/>
         <v>66.1738</v>
       </c>
-      <c r="R35" s="74" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="36" spans="1:18" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R35" s="71"/>
+    </row>
+    <row r="36" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="1"/>
       <c r="B36" s="53">
         <f>ROW(B36) - ROW($B$9)</f>
         <v>27</v>
       </c>
       <c r="C36" s="37" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="D36" s="37" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="E36" s="38" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="F36" s="37" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="G36" s="38" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="H36" s="37" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="I36" s="37" t="s">
-        <v>225</v>
+        <v>215</v>
       </c>
       <c r="J36" s="37" t="s">
-        <v>226</v>
+        <v>216</v>
       </c>
       <c r="K36" s="38" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="L36" s="37">
         <v>1</v>
       </c>
       <c r="M36" s="37">
-        <f t="shared" si="2"/>
+        <f>L36*20</f>
         <v>20</v>
       </c>
       <c r="N36" s="37">
         <v>22</v>
       </c>
       <c r="O36" s="60" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="P36" s="37">
         <v>4.2937000000000003</v>
@@ -3481,9 +3525,7 @@
         <f t="shared" si="1"/>
         <v>94.461400000000012</v>
       </c>
-      <c r="R36" s="72" t="s">
-        <v>227</v>
-      </c>
+      <c r="R36" s="69"/>
     </row>
     <row r="37" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="1"/>
@@ -3492,44 +3534,44 @@
         <v>28</v>
       </c>
       <c r="C37" s="39" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="D37" s="39" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="E37" s="40" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="F37" s="39" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="G37" s="40" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="H37" s="39" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="I37" s="39" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="J37" s="39" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="K37" s="40" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="L37" s="39">
         <v>1</v>
       </c>
       <c r="M37" s="39">
-        <f t="shared" si="2"/>
+        <f>L37*20</f>
         <v>20</v>
       </c>
       <c r="N37" s="39">
         <v>22</v>
       </c>
       <c r="O37" s="61" t="s">
-        <v>228</v>
+        <v>217</v>
       </c>
       <c r="P37" s="39">
         <v>10.6416</v>
@@ -3547,44 +3589,44 @@
         <v>29</v>
       </c>
       <c r="C38" s="37" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="D38" s="37" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="E38" s="38" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="F38" s="37" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="G38" s="38" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="H38" s="37" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="I38" s="37" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="J38" s="37" t="s">
-        <v>229</v>
+        <v>218</v>
       </c>
       <c r="K38" s="38" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="L38" s="37">
         <v>1</v>
       </c>
       <c r="M38" s="37">
-        <f t="shared" si="2"/>
+        <f>L38*20</f>
         <v>20</v>
       </c>
       <c r="N38" s="37">
         <v>22</v>
       </c>
       <c r="O38" s="60" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="P38" s="37">
         <v>0.3337</v>
@@ -3602,44 +3644,44 @@
         <v>30</v>
       </c>
       <c r="C39" s="39" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="D39" s="39" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="E39" s="40" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="F39" s="39" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="G39" s="40" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="H39" s="39" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="I39" s="39" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="J39" s="39" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="K39" s="40" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="L39" s="39">
         <v>1</v>
       </c>
       <c r="M39" s="39">
-        <f t="shared" si="2"/>
+        <f>L39*20</f>
         <v>20</v>
       </c>
       <c r="N39" s="39">
         <v>22</v>
       </c>
       <c r="O39" s="61" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="P39" s="39">
         <v>1.06</v>
@@ -3657,44 +3699,44 @@
         <v>31</v>
       </c>
       <c r="C40" s="37" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="D40" s="37" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="E40" s="38" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="F40" s="37" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="G40" s="38" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="H40" s="37" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="I40" s="37" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="J40" s="37" t="s">
-        <v>230</v>
+        <v>219</v>
       </c>
       <c r="K40" s="38" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="L40" s="37">
         <v>1</v>
       </c>
       <c r="M40" s="37">
-        <f t="shared" si="2"/>
+        <f>L40*20</f>
         <v>20</v>
       </c>
       <c r="N40" s="37">
         <v>22</v>
       </c>
       <c r="O40" s="60" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="P40" s="37">
         <v>0.77</v>
@@ -3712,44 +3754,44 @@
         <v>32</v>
       </c>
       <c r="C41" s="39" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="D41" s="39" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="E41" s="40" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="F41" s="39" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="G41" s="40" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="H41" s="39" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="I41" s="39" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="J41" s="39" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="K41" s="40" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="L41" s="39">
         <v>1</v>
       </c>
       <c r="M41" s="39">
-        <f t="shared" si="2"/>
+        <f>L41*20</f>
         <v>20</v>
       </c>
       <c r="N41" s="39">
         <v>22</v>
       </c>
       <c r="O41" s="61" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="P41" s="39">
         <v>0.499</v>
@@ -3767,44 +3809,44 @@
         <v>33</v>
       </c>
       <c r="C42" s="37" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="D42" s="37" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="E42" s="38" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="F42" s="37" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="G42" s="38" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="H42" s="37" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="I42" s="37" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="J42" s="58" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="K42" s="38" t="s">
-        <v>231</v>
+        <v>220</v>
       </c>
       <c r="L42" s="37">
         <v>1</v>
       </c>
       <c r="M42" s="37">
-        <f t="shared" si="2"/>
+        <f>L42*20</f>
         <v>20</v>
       </c>
       <c r="N42" s="37">
         <v>22</v>
       </c>
       <c r="O42" s="60" t="s">
-        <v>203</v>
+        <v>194</v>
       </c>
       <c r="P42" s="37">
         <v>0.69</v>
@@ -3833,12 +3875,12 @@
       <c r="M43" s="36"/>
       <c r="N43" s="36"/>
       <c r="O43" s="65" t="s">
-        <v>232</v>
+        <v>221</v>
       </c>
       <c r="P43" s="66"/>
       <c r="Q43" s="65">
         <f>SUM(Q10:Q42)</f>
-        <v>795.37520000000006</v>
+        <v>794.87919999999997</v>
       </c>
       <c r="R43" s="44"/>
     </row>
@@ -3860,12 +3902,12 @@
       <c r="M44" s="9"/>
       <c r="N44" s="9"/>
       <c r="O44" s="67" t="s">
-        <v>233</v>
+        <v>222</v>
       </c>
       <c r="P44" s="68"/>
       <c r="Q44" s="67">
         <f>Q43/20</f>
-        <v>39.76876</v>
+        <v>39.743960000000001</v>
       </c>
       <c r="R44" s="45"/>
     </row>
@@ -3881,35 +3923,34 @@
     <hyperlink ref="O13" r:id="rId4"/>
     <hyperlink ref="O14" r:id="rId5"/>
     <hyperlink ref="O15" r:id="rId6"/>
-    <hyperlink ref="O16" r:id="rId7"/>
-    <hyperlink ref="O17" r:id="rId8"/>
-    <hyperlink ref="O18" r:id="rId9"/>
-    <hyperlink ref="O19" r:id="rId10"/>
-    <hyperlink ref="O20" r:id="rId11"/>
-    <hyperlink ref="O21" r:id="rId12"/>
-    <hyperlink ref="O22" r:id="rId13"/>
-    <hyperlink ref="O23" r:id="rId14"/>
-    <hyperlink ref="O24" r:id="rId15"/>
-    <hyperlink ref="O25" r:id="rId16"/>
-    <hyperlink ref="O26" r:id="rId17"/>
-    <hyperlink ref="O27" r:id="rId18"/>
-    <hyperlink ref="O28" r:id="rId19"/>
-    <hyperlink ref="O29" r:id="rId20"/>
-    <hyperlink ref="O30" r:id="rId21"/>
-    <hyperlink ref="O31" r:id="rId22"/>
-    <hyperlink ref="O33" r:id="rId23"/>
-    <hyperlink ref="O34" r:id="rId24"/>
-    <hyperlink ref="O35" r:id="rId25"/>
-    <hyperlink ref="O36" r:id="rId26"/>
-    <hyperlink ref="O37" r:id="rId27"/>
-    <hyperlink ref="O38" r:id="rId28"/>
-    <hyperlink ref="O39" r:id="rId29"/>
-    <hyperlink ref="O40" r:id="rId30"/>
-    <hyperlink ref="O41" r:id="rId31"/>
-    <hyperlink ref="O42" r:id="rId32"/>
+    <hyperlink ref="O17" r:id="rId7"/>
+    <hyperlink ref="O18" r:id="rId8"/>
+    <hyperlink ref="O19" r:id="rId9"/>
+    <hyperlink ref="O20" r:id="rId10"/>
+    <hyperlink ref="O21" r:id="rId11"/>
+    <hyperlink ref="O22" r:id="rId12"/>
+    <hyperlink ref="O23" r:id="rId13"/>
+    <hyperlink ref="O24" r:id="rId14"/>
+    <hyperlink ref="O25" r:id="rId15"/>
+    <hyperlink ref="O26" r:id="rId16"/>
+    <hyperlink ref="O27" r:id="rId17"/>
+    <hyperlink ref="O28" r:id="rId18"/>
+    <hyperlink ref="O29" r:id="rId19"/>
+    <hyperlink ref="O30" r:id="rId20"/>
+    <hyperlink ref="O33" r:id="rId21"/>
+    <hyperlink ref="O34" r:id="rId22"/>
+    <hyperlink ref="O35" r:id="rId23"/>
+    <hyperlink ref="O36" r:id="rId24"/>
+    <hyperlink ref="O37" r:id="rId25"/>
+    <hyperlink ref="O38" r:id="rId26"/>
+    <hyperlink ref="O39" r:id="rId27"/>
+    <hyperlink ref="O40" r:id="rId28"/>
+    <hyperlink ref="O41" r:id="rId29"/>
+    <hyperlink ref="O42" r:id="rId30"/>
+    <hyperlink ref="O31" r:id="rId31"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId33"/>
-  <drawing r:id="rId34"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId32"/>
+  <drawing r:id="rId33"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
MCU variants added in Bottom Board BOM
</commit_message>
<xml_diff>
--- a/Deliverables/SM_Bottom Board/_BOM/eSpark BOM _Bottom (20 Boards).xlsx
+++ b/Deliverables/SM_Bottom Board/_BOM/eSpark BOM _Bottom (20 Boards).xlsx
@@ -5,7 +5,7 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Faizan\GitHub\ColeBenson-SmartMotors\Deliverables\SM_Bottom Board\_BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Faizan\GitHub\ColeBenson-SmartMotors\Deliverables\SM_Bottom Board\_BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -14,7 +14,7 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="152511"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="234">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="235">
   <si>
     <t>Component list</t>
   </si>
@@ -662,12 +662,6 @@
   </si>
   <si>
     <t>C778132</t>
-  </si>
-  <si>
-    <t>STM32F407VET6</t>
-  </si>
-  <si>
-    <t>C28730</t>
   </si>
   <si>
     <t>SN65HVDA1040AQDRQ1</t>
@@ -744,11 +738,20 @@
   <si>
     <t>C105588</t>
   </si>
+  <si>
+    <t>STM32F407VET6, STM32F407VET6</t>
+  </si>
+  <si>
+    <t>C12345, C28730</t>
+  </si>
+  <si>
+    <t>Multiple options added for MCU</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
   </numFmts>
@@ -1405,6 +1408,36 @@
     <xf numFmtId="0" fontId="20" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1413,36 +1446,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="4" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="15" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1488,7 +1491,7 @@
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1787,25 +1790,25 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:R44"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="3.140625" style="25" customWidth="1"/>
-    <col min="3" max="3" width="18.7109375" style="25" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="3.109375" style="25" customWidth="1"/>
+    <col min="3" max="3" width="18.6640625" style="25" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="36" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="30" customWidth="1"/>
-    <col min="6" max="6" width="26.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="33.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="33.42578125" customWidth="1"/>
-    <col min="11" max="11" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="20.85546875" customWidth="1"/>
-    <col min="14" max="15" width="19.140625" customWidth="1"/>
-    <col min="16" max="18" width="29.42578125" customWidth="1"/>
-    <col min="20" max="20" width="18.28515625" customWidth="1"/>
+    <col min="6" max="6" width="26.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="33.44140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.44140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="33.44140625" customWidth="1"/>
+    <col min="11" max="11" width="17.88671875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="20.88671875" customWidth="1"/>
+    <col min="14" max="15" width="19.109375" customWidth="1"/>
+    <col min="16" max="18" width="29.44140625" customWidth="1"/>
+    <col min="20" max="20" width="18.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1"/>
       <c r="B1" s="19"/>
       <c r="C1" s="19"/>
@@ -1816,16 +1819,16 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="72"/>
-      <c r="L1" s="72"/>
-      <c r="M1" s="72"/>
-      <c r="N1" s="72"/>
-      <c r="O1" s="72"/>
-      <c r="P1" s="72"/>
-      <c r="Q1" s="72"/>
-      <c r="R1" s="72"/>
-    </row>
-    <row r="2" spans="1:18" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K1" s="82"/>
+      <c r="L1" s="82"/>
+      <c r="M1" s="82"/>
+      <c r="N1" s="82"/>
+      <c r="O1" s="82"/>
+      <c r="P1" s="82"/>
+      <c r="Q1" s="82"/>
+      <c r="R1" s="82"/>
+    </row>
+    <row r="2" spans="1:18" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
       <c r="B2" s="20"/>
       <c r="C2" s="46"/>
@@ -1849,7 +1852,7 @@
       <c r="Q2" s="3"/>
       <c r="R2" s="43"/>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
       <c r="B3" s="21"/>
       <c r="C3" s="47"/>
@@ -1871,9 +1874,9 @@
       <c r="O3" s="4"/>
       <c r="P3" s="4"/>
       <c r="Q3" s="4"/>
-      <c r="R3" s="73"/>
-    </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="R3" s="83"/>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
       <c r="B4" s="21"/>
       <c r="C4" s="47"/>
@@ -1895,9 +1898,9 @@
       <c r="O4" s="6"/>
       <c r="P4" s="6"/>
       <c r="Q4" s="59"/>
-      <c r="R4" s="74"/>
-    </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="R4" s="84"/>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
       <c r="B5" s="21"/>
       <c r="C5" s="47"/>
@@ -1919,9 +1922,9 @@
       <c r="O5" s="5"/>
       <c r="P5" s="5"/>
       <c r="Q5" s="59"/>
-      <c r="R5" s="74"/>
-    </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="R5" s="84"/>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
       <c r="B6" s="22"/>
       <c r="C6" s="48"/>
@@ -1939,9 +1942,9 @@
       <c r="O6" s="5"/>
       <c r="P6" s="5"/>
       <c r="Q6" s="59"/>
-      <c r="R6" s="74"/>
-    </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="R6" s="84"/>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>
       <c r="B7" s="23"/>
       <c r="C7" s="49"/>
@@ -1959,9 +1962,9 @@
       <c r="O7" s="7"/>
       <c r="P7" s="7"/>
       <c r="Q7" s="7"/>
-      <c r="R7" s="74"/>
-    </row>
-    <row r="8" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R7" s="84"/>
+    </row>
+    <row r="8" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="1"/>
       <c r="B8" s="26"/>
       <c r="C8" s="50"/>
@@ -1979,9 +1982,9 @@
       <c r="O8" s="7"/>
       <c r="P8" s="7"/>
       <c r="Q8" s="7"/>
-      <c r="R8" s="74"/>
-    </row>
-    <row r="9" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R8" s="84"/>
+    </row>
+    <row r="9" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="1"/>
       <c r="B9" s="29" t="s">
         <v>4</v>
@@ -2035,7 +2038,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="10" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="1"/>
       <c r="B10" s="53">
         <f>ROW(B10) - ROW($B$9)</f>
@@ -2090,7 +2093,7 @@
       </c>
       <c r="R10" s="41"/>
     </row>
-    <row r="11" spans="1:18" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="1"/>
       <c r="B11" s="53">
         <f t="shared" ref="B11:B41" si="0">ROW(B11) - ROW($B$9)</f>
@@ -2100,7 +2103,7 @@
         <v>157</v>
       </c>
       <c r="D11" s="39" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="E11" s="40" t="s">
         <v>42</v>
@@ -2123,7 +2126,7 @@
       <c r="K11" s="40" t="s">
         <v>144</v>
       </c>
-      <c r="L11" s="76">
+      <c r="L11" s="73">
         <v>18</v>
       </c>
       <c r="M11" s="39">
@@ -2143,11 +2146,11 @@
         <f t="shared" ref="Q11:Q42" si="1">P11*N11</f>
         <v>0.55999999999999994</v>
       </c>
-      <c r="R11" s="79" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="12" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R11" s="76" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="1"/>
       <c r="B12" s="53">
         <f>ROW(B12) - ROW($B$9)</f>
@@ -2184,7 +2187,7 @@
         <v>1</v>
       </c>
       <c r="M12" s="37">
-        <f t="shared" ref="M12:M31" si="2">L12*20</f>
+        <f t="shared" ref="M12:M30" si="2">L12*20</f>
         <v>20</v>
       </c>
       <c r="N12" s="37">
@@ -2202,7 +2205,7 @@
       </c>
       <c r="R12" s="69"/>
     </row>
-    <row r="13" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="1"/>
       <c r="B13" s="53">
         <f t="shared" si="0"/>
@@ -2257,7 +2260,7 @@
       </c>
       <c r="R13" s="42"/>
     </row>
-    <row r="14" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="1"/>
       <c r="B14" s="53">
         <f>ROW(B14) - ROW($B$9)</f>
@@ -2312,7 +2315,7 @@
       </c>
       <c r="R14" s="41"/>
     </row>
-    <row r="15" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="1"/>
       <c r="B15" s="53">
         <f t="shared" si="0"/>
@@ -2367,7 +2370,7 @@
       </c>
       <c r="R15" s="42"/>
     </row>
-    <row r="16" spans="1:18" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="1"/>
       <c r="B16" s="53">
         <f t="shared" si="0"/>
@@ -2422,7 +2425,7 @@
       </c>
       <c r="R16" s="42"/>
     </row>
-    <row r="17" spans="1:18" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="1"/>
       <c r="B17" s="53">
         <f>ROW(B17) - ROW($B$9)</f>
@@ -2432,7 +2435,7 @@
         <v>158</v>
       </c>
       <c r="D17" s="37" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="E17" s="38" t="s">
         <v>47</v>
@@ -2477,7 +2480,7 @@
       </c>
       <c r="R17" s="69"/>
     </row>
-    <row r="18" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="1"/>
       <c r="B18" s="53">
         <f t="shared" si="0"/>
@@ -2532,7 +2535,7 @@
       </c>
       <c r="R18" s="42"/>
     </row>
-    <row r="19" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:18" ht="36.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="1"/>
       <c r="B19" s="53">
         <f>ROW(B19) - ROW($B$9)</f>
@@ -2587,7 +2590,7 @@
       </c>
       <c r="R19" s="41"/>
     </row>
-    <row r="20" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="1"/>
       <c r="B20" s="53">
         <f t="shared" si="0"/>
@@ -2642,7 +2645,7 @@
       </c>
       <c r="R20" s="42"/>
     </row>
-    <row r="21" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="1"/>
       <c r="B21" s="53">
         <f>ROW(B21) - ROW($B$9)</f>
@@ -2697,7 +2700,7 @@
       </c>
       <c r="R21" s="41"/>
     </row>
-    <row r="22" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="1"/>
       <c r="B22" s="53">
         <f t="shared" si="0"/>
@@ -2752,7 +2755,7 @@
       </c>
       <c r="R22" s="42"/>
     </row>
-    <row r="23" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A23" s="1"/>
       <c r="B23" s="53">
         <f>ROW(B23) - ROW($B$9)</f>
@@ -2807,7 +2810,7 @@
       </c>
       <c r="R23" s="41"/>
     </row>
-    <row r="24" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="1"/>
       <c r="B24" s="53">
         <f t="shared" si="0"/>
@@ -2862,7 +2865,7 @@
       </c>
       <c r="R24" s="42"/>
     </row>
-    <row r="25" spans="1:18" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:18" ht="48.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A25" s="1"/>
       <c r="B25" s="53">
         <f>ROW(B25) - ROW($B$9)</f>
@@ -2917,7 +2920,7 @@
       </c>
       <c r="R25" s="41"/>
     </row>
-    <row r="26" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A26" s="1"/>
       <c r="B26" s="53">
         <f t="shared" si="0"/>
@@ -2972,7 +2975,7 @@
       </c>
       <c r="R26" s="42"/>
     </row>
-    <row r="27" spans="1:18" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A27" s="1"/>
       <c r="B27" s="53">
         <f>ROW(B27) - ROW($B$9)</f>
@@ -3027,7 +3030,7 @@
       </c>
       <c r="R27" s="41"/>
     </row>
-    <row r="28" spans="1:18" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A28" s="1"/>
       <c r="B28" s="53">
         <f t="shared" si="0"/>
@@ -3082,7 +3085,7 @@
       </c>
       <c r="R28" s="42"/>
     </row>
-    <row r="29" spans="1:18" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:18" ht="24.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A29" s="1"/>
       <c r="B29" s="53">
         <f>ROW(B29) - ROW($B$9)</f>
@@ -3091,8 +3094,8 @@
       <c r="C29" s="37" t="s">
         <v>164</v>
       </c>
-      <c r="D29" s="77" t="s">
-        <v>229</v>
+      <c r="D29" s="74" t="s">
+        <v>227</v>
       </c>
       <c r="E29" s="38" t="s">
         <v>59</v>
@@ -3115,7 +3118,7 @@
       <c r="K29" s="38" t="s">
         <v>153</v>
       </c>
-      <c r="L29" s="78">
+      <c r="L29" s="75">
         <v>2</v>
       </c>
       <c r="M29" s="37">
@@ -3136,10 +3139,10 @@
         <v>0.13999999999999999</v>
       </c>
       <c r="R29" s="69" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="30" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="30" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A30" s="1"/>
       <c r="B30" s="53">
         <f t="shared" si="0"/>
@@ -3194,63 +3197,63 @@
       </c>
       <c r="R30" s="42"/>
     </row>
-    <row r="31" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A31" s="1"/>
       <c r="B31" s="53">
         <v>22</v>
       </c>
-      <c r="C31" s="80" t="s">
+      <c r="C31" s="77" t="s">
         <v>164</v>
       </c>
-      <c r="D31" s="75" t="s">
+      <c r="D31" s="72" t="s">
+        <v>223</v>
+      </c>
+      <c r="E31" s="78" t="s">
+        <v>229</v>
+      </c>
+      <c r="F31" s="72" t="s">
+        <v>86</v>
+      </c>
+      <c r="G31" s="78" t="s">
+        <v>224</v>
+      </c>
+      <c r="H31" s="72" t="s">
+        <v>124</v>
+      </c>
+      <c r="I31" s="77" t="s">
+        <v>179</v>
+      </c>
+      <c r="J31" s="77" t="s">
+        <v>231</v>
+      </c>
+      <c r="K31" s="78" t="s">
         <v>225</v>
       </c>
-      <c r="E31" s="81" t="s">
-        <v>231</v>
-      </c>
-      <c r="F31" s="75" t="s">
-        <v>86</v>
-      </c>
-      <c r="G31" s="81" t="s">
-        <v>226</v>
-      </c>
-      <c r="H31" s="75" t="s">
-        <v>124</v>
-      </c>
-      <c r="I31" s="80" t="s">
-        <v>179</v>
-      </c>
-      <c r="J31" s="80" t="s">
-        <v>233</v>
-      </c>
-      <c r="K31" s="81" t="s">
-        <v>227</v>
-      </c>
-      <c r="L31" s="75">
+      <c r="L31" s="72">
         <v>2</v>
       </c>
-      <c r="M31" s="75">
-        <f>L31*20</f>
+      <c r="M31" s="72">
+        <f t="shared" ref="M31:M42" si="3">L31*20</f>
         <v>40</v>
       </c>
-      <c r="N31" s="80">
+      <c r="N31" s="77">
         <v>100</v>
       </c>
-      <c r="O31" s="82" t="s">
+      <c r="O31" s="79" t="s">
         <v>181</v>
       </c>
-      <c r="P31" s="80">
+      <c r="P31" s="77">
         <v>1E-3</v>
       </c>
-      <c r="Q31" s="83">
+      <c r="Q31" s="80">
         <f>P31*N31</f>
         <v>0.1</v>
       </c>
-      <c r="R31" s="84" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="32" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R31" s="81" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="32" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A32" s="1"/>
       <c r="B32" s="53">
         <f>ROW(B32) - ROW($B$9)</f>
@@ -3287,7 +3290,7 @@
         <v>8</v>
       </c>
       <c r="M32" s="62">
-        <f>L32*20</f>
+        <f t="shared" si="3"/>
         <v>160</v>
       </c>
       <c r="N32" s="62">
@@ -3307,7 +3310,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="33" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A33" s="1"/>
       <c r="B33" s="53">
         <f t="shared" si="0"/>
@@ -3344,7 +3347,7 @@
         <v>1</v>
       </c>
       <c r="M33" s="39">
-        <f>L33*20</f>
+        <f t="shared" si="3"/>
         <v>20</v>
       </c>
       <c r="N33" s="39">
@@ -3362,7 +3365,7 @@
       </c>
       <c r="R33" s="71"/>
     </row>
-    <row r="34" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A34" s="1"/>
       <c r="B34" s="53">
         <f>ROW(B34) - ROW($B$9)</f>
@@ -3387,10 +3390,10 @@
         <v>135</v>
       </c>
       <c r="I34" s="37" t="s">
-        <v>211</v>
+        <v>232</v>
       </c>
       <c r="J34" s="37" t="s">
-        <v>212</v>
+        <v>233</v>
       </c>
       <c r="K34" s="38" t="s">
         <v>179</v>
@@ -3399,7 +3402,7 @@
         <v>1</v>
       </c>
       <c r="M34" s="37">
-        <f>L34*20</f>
+        <f t="shared" si="3"/>
         <v>20</v>
       </c>
       <c r="N34" s="37">
@@ -3415,9 +3418,11 @@
         <f t="shared" si="1"/>
         <v>240.84939999999997</v>
       </c>
-      <c r="R34" s="69"/>
-    </row>
-    <row r="35" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R34" s="69" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="35" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A35" s="1"/>
       <c r="B35" s="53">
         <f t="shared" si="0"/>
@@ -3442,10 +3447,10 @@
         <v>136</v>
       </c>
       <c r="I35" s="39" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="J35" s="39" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="K35" s="40" t="s">
         <v>179</v>
@@ -3454,7 +3459,7 @@
         <v>1</v>
       </c>
       <c r="M35" s="39">
-        <f>L35*20</f>
+        <f t="shared" si="3"/>
         <v>20</v>
       </c>
       <c r="N35" s="39">
@@ -3472,7 +3477,7 @@
       </c>
       <c r="R35" s="71"/>
     </row>
-    <row r="36" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A36" s="1"/>
       <c r="B36" s="53">
         <f>ROW(B36) - ROW($B$9)</f>
@@ -3497,10 +3502,10 @@
         <v>137</v>
       </c>
       <c r="I36" s="37" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="J36" s="37" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="K36" s="38" t="s">
         <v>179</v>
@@ -3509,7 +3514,7 @@
         <v>1</v>
       </c>
       <c r="M36" s="37">
-        <f>L36*20</f>
+        <f t="shared" si="3"/>
         <v>20</v>
       </c>
       <c r="N36" s="37">
@@ -3527,7 +3532,7 @@
       </c>
       <c r="R36" s="69"/>
     </row>
-    <row r="37" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A37" s="1"/>
       <c r="B37" s="53">
         <f t="shared" si="0"/>
@@ -3564,14 +3569,14 @@
         <v>1</v>
       </c>
       <c r="M37" s="39">
-        <f>L37*20</f>
+        <f t="shared" si="3"/>
         <v>20</v>
       </c>
       <c r="N37" s="39">
         <v>22</v>
       </c>
       <c r="O37" s="61" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="P37" s="39">
         <v>10.6416</v>
@@ -3582,7 +3587,7 @@
       </c>
       <c r="R37" s="42"/>
     </row>
-    <row r="38" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A38" s="1"/>
       <c r="B38" s="53">
         <f>ROW(B38) - ROW($B$9)</f>
@@ -3610,7 +3615,7 @@
         <v>179</v>
       </c>
       <c r="J38" s="37" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="K38" s="38" t="s">
         <v>179</v>
@@ -3619,7 +3624,7 @@
         <v>1</v>
       </c>
       <c r="M38" s="37">
-        <f>L38*20</f>
+        <f t="shared" si="3"/>
         <v>20</v>
       </c>
       <c r="N38" s="37">
@@ -3637,7 +3642,7 @@
       </c>
       <c r="R38" s="41"/>
     </row>
-    <row r="39" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A39" s="1"/>
       <c r="B39" s="53">
         <f t="shared" si="0"/>
@@ -3674,7 +3679,7 @@
         <v>1</v>
       </c>
       <c r="M39" s="39">
-        <f>L39*20</f>
+        <f t="shared" si="3"/>
         <v>20</v>
       </c>
       <c r="N39" s="39">
@@ -3692,7 +3697,7 @@
       </c>
       <c r="R39" s="42"/>
     </row>
-    <row r="40" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A40" s="1"/>
       <c r="B40" s="53">
         <f>ROW(B40) - ROW($B$9)</f>
@@ -3720,7 +3725,7 @@
         <v>179</v>
       </c>
       <c r="J40" s="37" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="K40" s="38" t="s">
         <v>179</v>
@@ -3729,7 +3734,7 @@
         <v>1</v>
       </c>
       <c r="M40" s="37">
-        <f>L40*20</f>
+        <f t="shared" si="3"/>
         <v>20</v>
       </c>
       <c r="N40" s="37">
@@ -3747,7 +3752,7 @@
       </c>
       <c r="R40" s="41"/>
     </row>
-    <row r="41" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A41" s="1"/>
       <c r="B41" s="53">
         <f t="shared" si="0"/>
@@ -3784,7 +3789,7 @@
         <v>1</v>
       </c>
       <c r="M41" s="39">
-        <f>L41*20</f>
+        <f t="shared" si="3"/>
         <v>20</v>
       </c>
       <c r="N41" s="39">
@@ -3802,7 +3807,7 @@
       </c>
       <c r="R41" s="42"/>
     </row>
-    <row r="42" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A42" s="1"/>
       <c r="B42" s="53">
         <f>ROW(B42) - ROW($B$9)</f>
@@ -3833,13 +3838,13 @@
         <v>179</v>
       </c>
       <c r="K42" s="38" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="L42" s="37">
         <v>1</v>
       </c>
       <c r="M42" s="37">
-        <f>L42*20</f>
+        <f t="shared" si="3"/>
         <v>20</v>
       </c>
       <c r="N42" s="37">
@@ -3857,7 +3862,7 @@
       </c>
       <c r="R42" s="41"/>
     </row>
-    <row r="43" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A43" s="1"/>
       <c r="B43" s="32"/>
       <c r="C43" s="51"/>
@@ -3875,7 +3880,7 @@
       <c r="M43" s="36"/>
       <c r="N43" s="36"/>
       <c r="O43" s="65" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="P43" s="66"/>
       <c r="Q43" s="65">
@@ -3884,7 +3889,7 @@
       </c>
       <c r="R43" s="44"/>
     </row>
-    <row r="44" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A44" s="1"/>
       <c r="B44" s="24"/>
       <c r="C44" s="52"/>
@@ -3902,7 +3907,7 @@
       <c r="M44" s="9"/>
       <c r="N44" s="9"/>
       <c r="O44" s="67" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="P44" s="68"/>
       <c r="Q44" s="67">

</xml_diff>